<commit_message>
Complete Gate 0 and expand build-agent guide
</commit_message>
<xml_diff>
--- a/outputs/4b7976f0-1820-4ffa-a191-bf7c7f79b010/Rimrooms_Campaign_Economy_v0.2.xlsx
+++ b/outputs/4b7976f0-1820-4ffa-a191-bf7c7f79b010/Rimrooms_Campaign_Economy_v0.2.xlsx
@@ -2,10 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Economy" sheetId="1" r:id="Rff2e395caf1c4fbb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Scenarios" sheetId="2" r:id="Ra14f4517cab549fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bulk Logistics" sheetId="3" r:id="Rcd577d3687c345f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Capital" sheetId="4" r:id="Racca1d47b2214592"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Economy" sheetId="1" r:id="R5547e6f4b1774270"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Scenarios" sheetId="2" r:id="R28d3f3c5255148ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bulk Logistics" sheetId="3" r:id="R53a1a24b56974702"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery &amp; Capital" sheetId="4" r:id="R3a73f3317acf444c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extended Cases" sheetId="5" r:id="Rcef147d392b2425f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -121,7 +122,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="29">
+  <x:fills count="38">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -263,6 +264,51 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9E5F2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9E5F2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9E5F2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="7">
     <x:border/>
@@ -303,7 +349,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="275">
+  <x:cellXfs count="373">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1049,6 +1095,282 @@
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="205" fontId="6" fillId="28" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="29" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="29" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="1" fillId="31" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="31" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="1" fillId="31" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="6" fillId="31" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="6" fillId="31" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="6" fillId="31" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="31" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="31" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="31" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="6" fillId="31" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="6" fillId="31" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="6" fillId="31" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="6" fillId="31" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="1" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="32" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="32" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="1" fillId="34" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="34" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="1" fillId="34" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="6" fillId="34" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="6" fillId="34" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="6" fillId="34" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="1" fillId="34" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="34" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="1" fillId="34" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="34" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="6" fillId="34" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="6" fillId="34" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="6" fillId="34" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="6" fillId="34" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="34" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="34" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="34" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="34" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="34" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="34" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="8" fillId="34" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="8" fillId="34" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="35" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="35" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="1" fillId="37" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="37" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="1" fillId="37" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="6" fillId="37" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="6" fillId="37" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="6" fillId="37" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="1" fillId="37" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="37" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="6" fillId="37" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="6" fillId="37" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="37" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="37" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="37" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="37" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="8" fillId="37" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="8" fillId="37" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
@@ -1309,7 +1631,7 @@
         <x:v>Value (USD unless noted)</x:v>
       </x:c>
       <x:c r="C6" s="69"/>
-      <x:c r="D6" s="262" t="str">
+      <x:c r="D6" s="350" t="str">
         <x:v>Explanation</x:v>
       </x:c>
       <x:c r="E6" s="10"/>
@@ -1487,7 +1809,7 @@
         <x:v>Ending Company Account</x:v>
       </x:c>
       <x:c r="B19" s="66" t="n">
-        <x:f>SUM(B7:B18)+B27</x:f>
+        <x:f>SUM(B7:B18)+B27+'Extended Cases'!$D$7+'Extended Cases'!$G$7+'Extended Cases'!$R$7</x:f>
         <x:v>53500000</x:v>
       </x:c>
       <x:c r="C19" s="65"/>
@@ -2219,17 +2541,17 @@
       <x:c r="I5" s="231"/>
     </x:row>
     <x:row r="6" ht="24" customHeight="1">
-      <x:c r="A6" s="263" t="str">
+      <x:c r="A6" s="351" t="str">
         <x:v>Thirty-day stage account outlook (USD)</x:v>
       </x:c>
-      <x:c r="B6" s="263"/>
-      <x:c r="C6" s="263"/>
-      <x:c r="D6" s="263"/>
-      <x:c r="E6" s="264"/>
-      <x:c r="F6" s="263"/>
-      <x:c r="G6" s="263"/>
-      <x:c r="H6" s="263"/>
-      <x:c r="I6" s="263"/>
+      <x:c r="B6" s="351"/>
+      <x:c r="C6" s="351"/>
+      <x:c r="D6" s="351"/>
+      <x:c r="E6" s="352"/>
+      <x:c r="F6" s="351"/>
+      <x:c r="G6" s="351"/>
+      <x:c r="H6" s="351"/>
+      <x:c r="I6" s="351"/>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
       <x:c r="A7" s="133" t="str">
@@ -2247,16 +2569,16 @@
       <x:c r="E7" s="133" t="str">
         <x:v>Downside paid contracts</x:v>
       </x:c>
-      <x:c r="F7" s="265" t="str">
+      <x:c r="F7" s="353" t="str">
         <x:v>No-contract close (USD)</x:v>
       </x:c>
-      <x:c r="G7" s="265" t="str">
+      <x:c r="G7" s="353" t="str">
         <x:v>Recovery close before funding (USD)</x:v>
       </x:c>
-      <x:c r="H7" s="265" t="str">
+      <x:c r="H7" s="353" t="str">
         <x:v>Approved milestone release (USD)</x:v>
       </x:c>
-      <x:c r="I7" s="265" t="str">
+      <x:c r="I7" s="353" t="str">
         <x:v>Recovery close after funding (USD)</x:v>
       </x:c>
     </x:row>
@@ -3163,7 +3485,7 @@
         <x:v>Closing account, planning</x:v>
       </x:c>
       <x:c r="C54" s="105" t="n">
-        <x:f>C43+C44+SUM(C45:C53)-'Recovery &amp; Capital'!$I$8</x:f>
+        <x:f>C43+C44+SUM(C45:C53)-'Recovery &amp; Capital'!$I$8+'Extended Cases'!$D$8+'Extended Cases'!$G$8+'Extended Cases'!$P$8-MIN(MAX(0,'Extended Cases'!$O$8),MAX(0,C44))</x:f>
         <x:v>56250000</x:v>
       </x:c>
       <x:c r="D54" s="41" t="str">
@@ -3217,7 +3539,7 @@
         <x:v>Closing account, downside</x:v>
       </x:c>
       <x:c r="C57" s="105" t="n">
-        <x:f>C55+C56+SUM(C45:C53)-'Recovery &amp; Capital'!$I$8</x:f>
+        <x:f>C55+C56+SUM(C45:C53)-'Recovery &amp; Capital'!$I$8+'Extended Cases'!$D$8+'Extended Cases'!$G$8+'Extended Cases'!$P$8-MIN(MAX(0,'Extended Cases'!$O$8),MAX(0,C56))</x:f>
         <x:v>48750000</x:v>
       </x:c>
       <x:c r="D57" s="41" t="str">
@@ -3671,7 +3993,7 @@
         <x:v>Closing account, planning</x:v>
       </x:c>
       <x:c r="C84" s="105" t="n">
-        <x:f>C73+C74+SUM(C75:C83)-'Recovery &amp; Capital'!$I$9</x:f>
+        <x:f>C73+C74+SUM(C75:C83)-'Recovery &amp; Capital'!$I$9+'Extended Cases'!$D$9+'Extended Cases'!$G$9+'Extended Cases'!$P$9-MIN(MAX(0,'Extended Cases'!$O$9),MAX(0,C74))</x:f>
         <x:v>81500000</x:v>
       </x:c>
       <x:c r="D84" s="41" t="str">
@@ -3725,7 +4047,7 @@
         <x:v>Closing account, downside</x:v>
       </x:c>
       <x:c r="C87" s="105" t="n">
-        <x:f>C85+C86+SUM(C75:C83)-'Recovery &amp; Capital'!$I$9</x:f>
+        <x:f>C85+C86+SUM(C75:C83)-'Recovery &amp; Capital'!$I$9+'Extended Cases'!$D$9+'Extended Cases'!$G$9+'Extended Cases'!$P$9-MIN(MAX(0,'Extended Cases'!$O$9),MAX(0,C86))</x:f>
         <x:v>54000000</x:v>
       </x:c>
       <x:c r="D87" s="41" t="str">
@@ -4179,7 +4501,7 @@
         <x:v>Closing account, planning</x:v>
       </x:c>
       <x:c r="C114" s="105" t="n">
-        <x:f>C103+C104+SUM(C105:C113)-'Recovery &amp; Capital'!$I$10</x:f>
+        <x:f>C103+C104+SUM(C105:C113)-'Recovery &amp; Capital'!$I$10+'Extended Cases'!$D$10+'Extended Cases'!$G$10+'Extended Cases'!$P$10-MIN(MAX(0,'Extended Cases'!$O$10),MAX(0,C104))</x:f>
         <x:v>169200000</x:v>
       </x:c>
       <x:c r="D114" s="41" t="str">
@@ -4233,7 +4555,7 @@
         <x:v>Closing account, downside</x:v>
       </x:c>
       <x:c r="C117" s="105" t="n">
-        <x:f>C115+C116+SUM(C105:C113)-'Recovery &amp; Capital'!$I$10</x:f>
+        <x:f>C115+C116+SUM(C105:C113)-'Recovery &amp; Capital'!$I$10+'Extended Cases'!$D$10+'Extended Cases'!$G$10+'Extended Cases'!$P$10-MIN(MAX(0,'Extended Cases'!$O$10),MAX(0,C116))</x:f>
         <x:v>91700000</x:v>
       </x:c>
       <x:c r="D117" s="41" t="str">
@@ -4687,7 +5009,7 @@
         <x:v>Closing account, planning</x:v>
       </x:c>
       <x:c r="C144" s="105" t="n">
-        <x:f>C133+C134+SUM(C135:C143)-'Recovery &amp; Capital'!$I$11</x:f>
+        <x:f>C133+C134+SUM(C135:C143)-'Recovery &amp; Capital'!$I$11+'Extended Cases'!$D$11+'Extended Cases'!$G$11+'Extended Cases'!$P$11-MIN(MAX(0,'Extended Cases'!$O$11),MAX(0,C134))</x:f>
         <x:v>518750000</x:v>
       </x:c>
       <x:c r="D144" s="41" t="str">
@@ -4741,7 +5063,7 @@
         <x:v>Closing account, downside</x:v>
       </x:c>
       <x:c r="C147" s="105" t="n">
-        <x:f>C145+C146+SUM(C135:C143)-'Recovery &amp; Capital'!$I$11</x:f>
+        <x:f>C145+C146+SUM(C135:C143)-'Recovery &amp; Capital'!$I$11+'Extended Cases'!$D$11+'Extended Cases'!$G$11+'Extended Cases'!$P$11-MIN(MAX(0,'Extended Cases'!$O$11),MAX(0,C146))</x:f>
         <x:v>216250000</x:v>
       </x:c>
       <x:c r="D147" s="41" t="str">
@@ -5195,7 +5517,7 @@
         <x:v>Closing account, planning</x:v>
       </x:c>
       <x:c r="C174" s="105" t="n">
-        <x:f>C163+C164+SUM(C165:C173)-'Recovery &amp; Capital'!$I$12</x:f>
+        <x:f>C163+C164+SUM(C165:C173)-'Recovery &amp; Capital'!$I$12+'Extended Cases'!$D$12+'Extended Cases'!$G$12+'Extended Cases'!$P$12-MIN(MAX(0,'Extended Cases'!$O$12),MAX(0,C164))</x:f>
         <x:v>1203500000</x:v>
       </x:c>
       <x:c r="D174" s="41" t="str">
@@ -5249,7 +5571,7 @@
         <x:v>Closing account, downside</x:v>
       </x:c>
       <x:c r="C177" s="105" t="n">
-        <x:f>C175+C176+SUM(C165:C173)-'Recovery &amp; Capital'!$I$12</x:f>
+        <x:f>C175+C176+SUM(C165:C173)-'Recovery &amp; Capital'!$I$12+'Extended Cases'!$D$12+'Extended Cases'!$G$12+'Extended Cases'!$P$12-MIN(MAX(0,'Extended Cases'!$O$12),MAX(0,C176))</x:f>
         <x:v>451000000</x:v>
       </x:c>
       <x:c r="D177" s="41" t="str">
@@ -5703,7 +6025,7 @@
         <x:v>Closing account, planning</x:v>
       </x:c>
       <x:c r="C204" s="105" t="n">
-        <x:f>C193+C194+SUM(C195:C203)-'Recovery &amp; Capital'!$I$13</x:f>
+        <x:f>C193+C194+SUM(C195:C203)-'Recovery &amp; Capital'!$I$13+'Extended Cases'!$D$13+'Extended Cases'!$G$13+'Extended Cases'!$P$13-MIN(MAX(0,'Extended Cases'!$O$13),MAX(0,C194))</x:f>
         <x:v>2285000000</x:v>
       </x:c>
       <x:c r="D204" s="41" t="str">
@@ -5757,7 +6079,7 @@
         <x:v>Closing account, downside</x:v>
       </x:c>
       <x:c r="C207" s="105" t="n">
-        <x:f>C205+C206+SUM(C195:C203)-'Recovery &amp; Capital'!$I$13</x:f>
+        <x:f>C205+C206+SUM(C195:C203)-'Recovery &amp; Capital'!$I$13+'Extended Cases'!$D$13+'Extended Cases'!$G$13+'Extended Cases'!$P$13-MIN(MAX(0,'Extended Cases'!$O$13),MAX(0,C206))</x:f>
         <x:v>632500000</x:v>
       </x:c>
       <x:c r="D207" s="41" t="str">
@@ -6188,86 +6510,86 @@
       <x:c r="N4" s="251"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="263" t="str">
+      <x:c r="A5" s="351" t="str">
         <x:v>Added monthly cost inputs</x:v>
       </x:c>
-      <x:c r="B5" s="263"/>
-      <x:c r="C5" s="263"/>
-      <x:c r="D5" s="263"/>
-      <x:c r="E5" s="263"/>
-      <x:c r="F5" s="263"/>
-      <x:c r="G5" s="263"/>
-      <x:c r="H5" s="263"/>
-      <x:c r="I5" s="263"/>
-      <x:c r="J5" s="263"/>
-      <x:c r="K5" s="263"/>
-      <x:c r="L5" s="263"/>
-      <x:c r="M5" s="263"/>
-      <x:c r="N5" s="263"/>
+      <x:c r="B5" s="351"/>
+      <x:c r="C5" s="351"/>
+      <x:c r="D5" s="351"/>
+      <x:c r="E5" s="351"/>
+      <x:c r="F5" s="351"/>
+      <x:c r="G5" s="351"/>
+      <x:c r="H5" s="351"/>
+      <x:c r="I5" s="351"/>
+      <x:c r="J5" s="351"/>
+      <x:c r="K5" s="351"/>
+      <x:c r="L5" s="351"/>
+      <x:c r="M5" s="351"/>
+      <x:c r="N5" s="351"/>
     </x:row>
     <x:row r="6" ht="48" customHeight="1">
-      <x:c r="A6" s="268" t="str">
+      <x:c r="A6" s="356" t="str">
         <x:v>Campaign stage</x:v>
       </x:c>
-      <x:c r="B6" s="268" t="str">
+      <x:c r="B6" s="356" t="str">
         <x:v>Specialists (FTE)</x:v>
       </x:c>
-      <x:c r="C6" s="268" t="str">
+      <x:c r="C6" s="356" t="str">
         <x:v>Premium / specialist / day (USD)</x:v>
       </x:c>
-      <x:c r="D6" s="268" t="str">
+      <x:c r="D6" s="356" t="str">
         <x:v>Transport runs / month</x:v>
       </x:c>
-      <x:c r="E6" s="268" t="str">
+      <x:c r="E6" s="356" t="str">
         <x:v>Quoted transport / run (USD)</x:v>
       </x:c>
-      <x:c r="F6" s="268" t="str">
+      <x:c r="F6" s="356" t="str">
         <x:v>Equipment replacement quotes (USD / month)</x:v>
       </x:c>
-      <x:c r="G6" s="268" t="str">
+      <x:c r="G6" s="356" t="str">
         <x:v>Cargo replacement purchases (USD / month)</x:v>
       </x:c>
-      <x:c r="H6" s="268" t="str">
+      <x:c r="H6" s="356" t="str">
         <x:v>Security and site maintenance quote (USD / month)</x:v>
       </x:c>
-      <x:c r="I6" s="268" t="str">
+      <x:c r="I6" s="356" t="str">
         <x:v>Added monthly cost (USD)</x:v>
       </x:c>
-      <x:c r="J6" s="268" t="str">
+      <x:c r="J6" s="356" t="str">
         <x:v>Basis / status</x:v>
       </x:c>
-      <x:c r="K6" s="265"/>
-      <x:c r="L6" s="265"/>
-      <x:c r="M6" s="265"/>
-      <x:c r="N6" s="265"/>
+      <x:c r="K6" s="353"/>
+      <x:c r="L6" s="353"/>
+      <x:c r="M6" s="353"/>
+      <x:c r="N6" s="353"/>
     </x:row>
     <x:row r="7" ht="34" customHeight="1">
       <x:c r="A7" s="165" t="str">
         <x:v>Stage 1: First safe survey</x:v>
       </x:c>
-      <x:c r="B7" s="272" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C7" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D7" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E7" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F7" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G7" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H7" s="273" t="n">
+      <x:c r="B7" s="360" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C7" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D7" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E7" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F7" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G7" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H7" s="361" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I7" s="169" t="n">
-        <x:f>B7*C7*'Economy'!$C$32+D7*E7+SUM(F7:H7)</x:f>
+        <x:f>B7*C7*'Economy'!$C$32+D7*E7+SUM(F7:H7)+'Extended Cases'!$K$7+'Extended Cases'!$N$7+'Extended Cases'!$K$18+'Extended Cases'!$L$29</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="J7" s="170" t="str">
@@ -6282,29 +6604,29 @@
       <x:c r="A8" s="165" t="str">
         <x:v>Stage 2: Repeat access</x:v>
       </x:c>
-      <x:c r="B8" s="272" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C8" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D8" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E8" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F8" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G8" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H8" s="273" t="n">
+      <x:c r="B8" s="360" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C8" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D8" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E8" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F8" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G8" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H8" s="361" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I8" s="169" t="n">
-        <x:f>B8*C8*'Campaign Scenarios'!$C$32+D8*E8+SUM(F8:H8)</x:f>
+        <x:f>B8*C8*'Campaign Scenarios'!$C$32+D8*E8+SUM(F8:H8)+'Extended Cases'!$K$8+'Extended Cases'!$N$8+'Extended Cases'!$K$19+'Extended Cases'!$L$30</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="J8" s="170" t="str">
@@ -6319,29 +6641,29 @@
       <x:c r="A9" s="165" t="str">
         <x:v>Stage 3: Specialist services</x:v>
       </x:c>
-      <x:c r="B9" s="272" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C9" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D9" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E9" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F9" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G9" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H9" s="273" t="n">
+      <x:c r="B9" s="360" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C9" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D9" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E9" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F9" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G9" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H9" s="361" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I9" s="169" t="n">
-        <x:f>B9*C9*'Campaign Scenarios'!$C$62+D9*E9+SUM(F9:H9)</x:f>
+        <x:f>B9*C9*'Campaign Scenarios'!$C$62+D9*E9+SUM(F9:H9)+'Extended Cases'!$K$9+'Extended Cases'!$N$9+'Extended Cases'!$K$20+'Extended Cases'!$L$31</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="J9" s="170" t="str">
@@ -6356,29 +6678,29 @@
       <x:c r="A10" s="165" t="str">
         <x:v>Stage 4: Leases and remote sites</x:v>
       </x:c>
-      <x:c r="B10" s="272" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C10" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D10" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E10" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F10" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G10" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H10" s="273" t="n">
+      <x:c r="B10" s="360" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C10" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D10" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E10" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F10" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G10" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H10" s="361" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I10" s="169" t="n">
-        <x:f>B10*C10*'Campaign Scenarios'!$C$92+D10*E10+SUM(F10:H10)</x:f>
+        <x:f>B10*C10*'Campaign Scenarios'!$C$92+D10*E10+SUM(F10:H10)+'Extended Cases'!$K$10+'Extended Cases'!$N$10+'Extended Cases'!$K$21+'Extended Cases'!$L$32</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="J10" s="170" t="str">
@@ -6393,29 +6715,29 @@
       <x:c r="A11" s="165" t="str">
         <x:v>Stage 5: Large recovery and network work</x:v>
       </x:c>
-      <x:c r="B11" s="272" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C11" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D11" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E11" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F11" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G11" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H11" s="273" t="n">
+      <x:c r="B11" s="360" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C11" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D11" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E11" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F11" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G11" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H11" s="361" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I11" s="169" t="n">
-        <x:f>B11*C11*'Campaign Scenarios'!$C$122+D11*E11+SUM(F11:H11)</x:f>
+        <x:f>B11*C11*'Campaign Scenarios'!$C$122+D11*E11+SUM(F11:H11)+'Extended Cases'!$K$11+'Extended Cases'!$N$11+'Extended Cases'!$K$22+'Extended Cases'!$L$33</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="J11" s="170" t="str">
@@ -6430,29 +6752,29 @@
       <x:c r="A12" s="165" t="str">
         <x:v>Stage 6: Vehicle and optional orbital support</x:v>
       </x:c>
-      <x:c r="B12" s="272" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C12" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D12" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E12" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F12" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G12" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H12" s="273" t="n">
+      <x:c r="B12" s="360" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C12" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D12" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E12" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F12" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G12" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H12" s="361" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I12" s="169" t="n">
-        <x:f>B12*C12*'Campaign Scenarios'!$C$152+D12*E12+SUM(F12:H12)</x:f>
+        <x:f>B12*C12*'Campaign Scenarios'!$C$152+D12*E12+SUM(F12:H12)+'Extended Cases'!$K$12+'Extended Cases'!$N$12+'Extended Cases'!$K$23+'Extended Cases'!$L$34</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="J12" s="170" t="str">
@@ -6467,29 +6789,29 @@
       <x:c r="A13" s="165" t="str">
         <x:v>Stage 7: Deep-site operations</x:v>
       </x:c>
-      <x:c r="B13" s="272" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C13" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D13" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E13" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F13" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G13" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H13" s="273" t="n">
+      <x:c r="B13" s="360" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C13" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D13" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E13" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F13" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G13" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H13" s="361" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I13" s="169" t="n">
-        <x:f>B13*C13*'Campaign Scenarios'!$C$182+D13*E13+SUM(F13:H13)</x:f>
+        <x:f>B13*C13*'Campaign Scenarios'!$C$182+D13*E13+SUM(F13:H13)+'Extended Cases'!$K$13+'Extended Cases'!$N$13+'Extended Cases'!$K$24+'Extended Cases'!$L$35</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="J13" s="170" t="str">
@@ -6517,52 +6839,52 @@
       <x:c r="N14" s="10"/>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="263" t="str">
+      <x:c r="A15" s="351" t="str">
         <x:v>Milestone capital request controls</x:v>
       </x:c>
-      <x:c r="B15" s="263"/>
-      <x:c r="C15" s="263"/>
-      <x:c r="D15" s="263"/>
-      <x:c r="E15" s="263"/>
-      <x:c r="F15" s="263"/>
-      <x:c r="G15" s="263"/>
-      <x:c r="H15" s="263"/>
-      <x:c r="I15" s="263"/>
-      <x:c r="J15" s="263"/>
-      <x:c r="K15" s="263"/>
-      <x:c r="L15" s="263"/>
-      <x:c r="M15" s="263"/>
-      <x:c r="N15" s="263"/>
+      <x:c r="B15" s="351"/>
+      <x:c r="C15" s="351"/>
+      <x:c r="D15" s="351"/>
+      <x:c r="E15" s="351"/>
+      <x:c r="F15" s="351"/>
+      <x:c r="G15" s="351"/>
+      <x:c r="H15" s="351"/>
+      <x:c r="I15" s="351"/>
+      <x:c r="J15" s="351"/>
+      <x:c r="K15" s="351"/>
+      <x:c r="L15" s="351"/>
+      <x:c r="M15" s="351"/>
+      <x:c r="N15" s="351"/>
     </x:row>
     <x:row r="16" ht="44" customHeight="1">
-      <x:c r="A16" s="268" t="str">
+      <x:c r="A16" s="356" t="str">
         <x:v>Campaign stage</x:v>
       </x:c>
-      <x:c r="B16" s="268" t="str">
+      <x:c r="B16" s="356" t="str">
         <x:v>Candidate milestone (original game design)</x:v>
       </x:c>
-      <x:c r="C16" s="268" t="str">
+      <x:c r="C16" s="356" t="str">
         <x:v>Illustrative request target (USD)</x:v>
       </x:c>
-      <x:c r="D16" s="268" t="str">
+      <x:c r="D16" s="356" t="str">
         <x:v>Milestone achieved? (0/1)</x:v>
       </x:c>
-      <x:c r="E16" s="268" t="str">
+      <x:c r="E16" s="356" t="str">
         <x:v>Explicit approval? (0/1)</x:v>
       </x:c>
-      <x:c r="F16" s="268" t="str">
+      <x:c r="F16" s="356" t="str">
         <x:v>Release if both gates pass (USD)</x:v>
       </x:c>
-      <x:c r="G16" s="268" t="str">
+      <x:c r="G16" s="356" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="H16" s="265"/>
-      <x:c r="I16" s="265"/>
-      <x:c r="J16" s="265"/>
-      <x:c r="K16" s="265"/>
-      <x:c r="L16" s="265"/>
-      <x:c r="M16" s="265"/>
-      <x:c r="N16" s="265"/>
+      <x:c r="H16" s="353"/>
+      <x:c r="I16" s="353"/>
+      <x:c r="J16" s="353"/>
+      <x:c r="K16" s="353"/>
+      <x:c r="L16" s="353"/>
+      <x:c r="M16" s="353"/>
+      <x:c r="N16" s="353"/>
     </x:row>
     <x:row r="17" ht="56" customHeight="1">
       <x:c r="A17" s="165" t="str">
@@ -6571,13 +6893,13 @@
       <x:c r="B17" s="187" t="str">
         <x:v>Accepted first survey records and returned crew</x:v>
       </x:c>
-      <x:c r="C17" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D17" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E17" s="274" t="n">
+      <x:c r="C17" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D17" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E17" s="362" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F17" s="169" t="n">
@@ -6602,13 +6924,13 @@
       <x:c r="B18" s="187" t="str">
         <x:v>Three routes verified; equipment and cargo reconciled</x:v>
       </x:c>
-      <x:c r="C18" s="273" t="n">
+      <x:c r="C18" s="361" t="n">
         <x:v>25000000</x:v>
       </x:c>
-      <x:c r="D18" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E18" s="274" t="n">
+      <x:c r="D18" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E18" s="362" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F18" s="169" t="n">
@@ -6633,13 +6955,13 @@
       <x:c r="B19" s="187" t="str">
         <x:v>Usable sample analysis or specialist deliverable accepted</x:v>
       </x:c>
-      <x:c r="C19" s="273" t="n">
+      <x:c r="C19" s="361" t="n">
         <x:v>50000000</x:v>
       </x:c>
-      <x:c r="D19" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E19" s="274" t="n">
+      <x:c r="D19" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E19" s="362" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F19" s="169" t="n">
@@ -6664,13 +6986,13 @@
       <x:c r="B20" s="187" t="str">
         <x:v>Relay or outpost operating; evacuation route demonstrated</x:v>
       </x:c>
-      <x:c r="C20" s="273" t="n">
+      <x:c r="C20" s="361" t="n">
         <x:v>100000000</x:v>
       </x:c>
-      <x:c r="D20" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E20" s="274" t="n">
+      <x:c r="D20" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E20" s="362" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F20" s="169" t="n">
@@ -6695,13 +7017,13 @@
       <x:c r="B21" s="187" t="str">
         <x:v>Town response or large recovery closed with staff and cargo reconciled</x:v>
       </x:c>
-      <x:c r="C21" s="273" t="n">
+      <x:c r="C21" s="361" t="n">
         <x:v>250000000</x:v>
       </x:c>
-      <x:c r="D21" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E21" s="274" t="n">
+      <x:c r="D21" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E21" s="362" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F21" s="169" t="n">
@@ -6726,13 +7048,13 @@
       <x:c r="B22" s="187" t="str">
         <x:v>Transport or gravship logistics test completed with cargo records</x:v>
       </x:c>
-      <x:c r="C22" s="273" t="n">
+      <x:c r="C22" s="361" t="n">
         <x:v>500000000</x:v>
       </x:c>
-      <x:c r="D22" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E22" s="274" t="n">
+      <x:c r="D22" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E22" s="362" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F22" s="169" t="n">
@@ -6757,13 +7079,13 @@
       <x:c r="B23" s="187" t="str">
         <x:v>Deep-site objective returned with route and containment records</x:v>
       </x:c>
-      <x:c r="C23" s="273" t="n">
+      <x:c r="C23" s="361" t="n">
         <x:v>1000000000</x:v>
       </x:c>
-      <x:c r="D23" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E23" s="274" t="n">
+      <x:c r="D23" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E23" s="362" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F23" s="169" t="n">
@@ -6798,22 +7120,22 @@
       <x:c r="N24" s="10"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="263" t="str">
+      <x:c r="A25" s="351" t="str">
         <x:v>No-contract recovery actions</x:v>
       </x:c>
-      <x:c r="B25" s="263"/>
-      <x:c r="C25" s="263"/>
-      <x:c r="D25" s="263"/>
-      <x:c r="E25" s="263"/>
-      <x:c r="F25" s="263"/>
-      <x:c r="G25" s="263"/>
-      <x:c r="H25" s="263"/>
-      <x:c r="I25" s="263"/>
-      <x:c r="J25" s="263"/>
-      <x:c r="K25" s="263"/>
-      <x:c r="L25" s="263"/>
-      <x:c r="M25" s="263"/>
-      <x:c r="N25" s="263"/>
+      <x:c r="B25" s="351"/>
+      <x:c r="C25" s="351"/>
+      <x:c r="D25" s="351"/>
+      <x:c r="E25" s="351"/>
+      <x:c r="F25" s="351"/>
+      <x:c r="G25" s="351"/>
+      <x:c r="H25" s="351"/>
+      <x:c r="I25" s="351"/>
+      <x:c r="J25" s="351"/>
+      <x:c r="K25" s="351"/>
+      <x:c r="L25" s="351"/>
+      <x:c r="M25" s="351"/>
+      <x:c r="N25" s="351"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="52" t="str">
@@ -6834,46 +7156,46 @@
       <x:c r="N26" s="52"/>
     </x:row>
     <x:row r="27" ht="58" customHeight="1">
-      <x:c r="A27" s="268" t="str">
+      <x:c r="A27" s="356" t="str">
         <x:v>Campaign stage</x:v>
       </x:c>
-      <x:c r="B27" s="268" t="str">
+      <x:c r="B27" s="356" t="str">
         <x:v>Retained payroll headcount</x:v>
       </x:c>
-      <x:c r="C27" s="268" t="str">
+      <x:c r="C27" s="356" t="str">
         <x:v>Specialists retained (FTE)</x:v>
       </x:c>
-      <x:c r="D27" s="268" t="str">
+      <x:c r="D27" s="356" t="str">
         <x:v>Additional hires approved</x:v>
       </x:c>
-      <x:c r="E27" s="268" t="str">
+      <x:c r="E27" s="356" t="str">
         <x:v>Outpost service days retained</x:v>
       </x:c>
-      <x:c r="F27" s="268" t="str">
+      <x:c r="F27" s="356" t="str">
         <x:v>Extra facility lease days retained</x:v>
       </x:c>
-      <x:c r="G27" s="268" t="str">
+      <x:c r="G27" s="356" t="str">
         <x:v>Survey-kit orders</x:v>
       </x:c>
-      <x:c r="H27" s="268" t="str">
+      <x:c r="H27" s="356" t="str">
         <x:v>Research-material orders</x:v>
       </x:c>
-      <x:c r="I27" s="268" t="str">
+      <x:c r="I27" s="356" t="str">
         <x:v>Transport runs</x:v>
       </x:c>
-      <x:c r="J27" s="268" t="str">
+      <x:c r="J27" s="356" t="str">
         <x:v>Equipment replacement quote (USD)</x:v>
       </x:c>
-      <x:c r="K27" s="268" t="str">
+      <x:c r="K27" s="356" t="str">
         <x:v>Cargo replacement purchases (USD)</x:v>
       </x:c>
-      <x:c r="L27" s="268" t="str">
+      <x:c r="L27" s="356" t="str">
         <x:v>Security / maintenance quote (USD)</x:v>
       </x:c>
-      <x:c r="M27" s="268" t="str">
+      <x:c r="M27" s="356" t="str">
         <x:v>Other committed quote (USD)</x:v>
       </x:c>
-      <x:c r="N27" s="268" t="str">
+      <x:c r="N27" s="356" t="str">
         <x:v>Basis / status</x:v>
       </x:c>
     </x:row>
@@ -6881,40 +7203,40 @@
       <x:c r="A28" s="165" t="str">
         <x:v>Stage 1: First safe survey</x:v>
       </x:c>
-      <x:c r="B28" s="274" t="n">
+      <x:c r="B28" s="362" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C28" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D28" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E28" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F28" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G28" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H28" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I28" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J28" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K28" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L28" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M28" s="273" t="n">
+      <x:c r="C28" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D28" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E28" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F28" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G28" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H28" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I28" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J28" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K28" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L28" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M28" s="361" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N28" s="170" t="str">
@@ -6925,40 +7247,40 @@
       <x:c r="A29" s="165" t="str">
         <x:v>Stage 2: Repeat access</x:v>
       </x:c>
-      <x:c r="B29" s="274" t="n">
+      <x:c r="B29" s="362" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C29" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D29" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E29" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F29" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G29" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H29" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I29" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J29" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K29" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L29" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M29" s="273" t="n">
+      <x:c r="C29" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D29" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E29" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F29" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G29" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H29" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I29" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J29" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K29" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L29" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M29" s="361" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N29" s="170" t="str">
@@ -6969,40 +7291,40 @@
       <x:c r="A30" s="165" t="str">
         <x:v>Stage 3: Specialist services</x:v>
       </x:c>
-      <x:c r="B30" s="274" t="n">
+      <x:c r="B30" s="362" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C30" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D30" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E30" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F30" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G30" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H30" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I30" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J30" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K30" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L30" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M30" s="273" t="n">
+      <x:c r="C30" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D30" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E30" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F30" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G30" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H30" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I30" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J30" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K30" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L30" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M30" s="361" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N30" s="170" t="str">
@@ -7013,40 +7335,40 @@
       <x:c r="A31" s="165" t="str">
         <x:v>Stage 4: Leases and remote sites</x:v>
       </x:c>
-      <x:c r="B31" s="274" t="n">
+      <x:c r="B31" s="362" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="C31" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D31" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E31" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F31" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G31" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H31" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I31" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J31" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K31" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L31" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M31" s="273" t="n">
+      <x:c r="C31" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D31" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E31" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F31" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G31" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H31" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I31" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J31" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K31" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L31" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M31" s="361" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N31" s="170" t="str">
@@ -7057,40 +7379,40 @@
       <x:c r="A32" s="165" t="str">
         <x:v>Stage 5: Large recovery and network work</x:v>
       </x:c>
-      <x:c r="B32" s="274" t="n">
+      <x:c r="B32" s="362" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="C32" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D32" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E32" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F32" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G32" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H32" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I32" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J32" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K32" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L32" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M32" s="273" t="n">
+      <x:c r="C32" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D32" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E32" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F32" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G32" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H32" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I32" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J32" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K32" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L32" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M32" s="361" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N32" s="170" t="str">
@@ -7101,40 +7423,40 @@
       <x:c r="A33" s="165" t="str">
         <x:v>Stage 6: Vehicle and optional orbital support</x:v>
       </x:c>
-      <x:c r="B33" s="274" t="n">
+      <x:c r="B33" s="362" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C33" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D33" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E33" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F33" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G33" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H33" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I33" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J33" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K33" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L33" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M33" s="273" t="n">
+      <x:c r="C33" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D33" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E33" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F33" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G33" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H33" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I33" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J33" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K33" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L33" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M33" s="361" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N33" s="170" t="str">
@@ -7145,40 +7467,40 @@
       <x:c r="A34" s="165" t="str">
         <x:v>Stage 7: Deep-site operations</x:v>
       </x:c>
-      <x:c r="B34" s="274" t="n">
+      <x:c r="B34" s="362" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C34" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D34" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E34" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F34" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G34" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H34" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I34" s="274" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J34" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K34" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L34" s="273" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M34" s="273" t="n">
+      <x:c r="C34" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D34" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E34" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F34" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G34" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H34" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I34" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J34" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K34" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L34" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M34" s="361" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="N34" s="170" t="str">
@@ -7202,26 +7524,26 @@
       <x:c r="N35" s="10"/>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="263" t="str">
+      <x:c r="A36" s="351" t="str">
         <x:v>Monthly stage case bridge (USD)</x:v>
       </x:c>
-      <x:c r="B36" s="263"/>
-      <x:c r="C36" s="263"/>
-      <x:c r="D36" s="263"/>
-      <x:c r="E36" s="263"/>
-      <x:c r="F36" s="263"/>
-      <x:c r="G36" s="263"/>
-      <x:c r="H36" s="263"/>
-      <x:c r="I36" s="263"/>
-      <x:c r="J36" s="263"/>
-      <x:c r="K36" s="263"/>
-      <x:c r="L36" s="263"/>
-      <x:c r="M36" s="263"/>
-      <x:c r="N36" s="263"/>
+      <x:c r="B36" s="351"/>
+      <x:c r="C36" s="351"/>
+      <x:c r="D36" s="351"/>
+      <x:c r="E36" s="351"/>
+      <x:c r="F36" s="351"/>
+      <x:c r="G36" s="351"/>
+      <x:c r="H36" s="351"/>
+      <x:c r="I36" s="351"/>
+      <x:c r="J36" s="351"/>
+      <x:c r="K36" s="351"/>
+      <x:c r="L36" s="351"/>
+      <x:c r="M36" s="351"/>
+      <x:c r="N36" s="351"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="52" t="str">
-        <x:v>No-contract removes this month’s planned receipts. Recovery applies the controls above. A parent-company release needs both recorded milestone completion and explicit approval.</x:v>
+        <x:v>No-new-contract removes contract receipts. Delivered services, earned leases, and accepted claims count only when entered. Recovery applies actual commitments above and below; funding needs both milestone completion and explicit approval.</x:v>
       </x:c>
       <x:c r="B37" s="52"/>
       <x:c r="C37" s="52"/>
@@ -7238,40 +7560,40 @@
       <x:c r="N37" s="10"/>
     </x:row>
     <x:row r="38" ht="50" customHeight="1">
-      <x:c r="A38" s="268" t="str">
+      <x:c r="A38" s="356" t="str">
         <x:v>Campaign stage</x:v>
       </x:c>
-      <x:c r="B38" s="268" t="str">
+      <x:c r="B38" s="356" t="str">
         <x:v>Opening balance on base path</x:v>
       </x:c>
-      <x:c r="C38" s="268" t="str">
-        <x:v>Planned case receipts</x:v>
-      </x:c>
-      <x:c r="D38" s="268" t="str">
-        <x:v>Planned case costs, including new quotes</x:v>
-      </x:c>
-      <x:c r="E38" s="268" t="str">
-        <x:v>No-contract month close</x:v>
-      </x:c>
-      <x:c r="F38" s="268" t="str">
+      <x:c r="C38" s="356" t="str">
+        <x:v>Planned receipts: contracts + services + leases + claims</x:v>
+      </x:c>
+      <x:c r="D38" s="356" t="str">
+        <x:v>Planned costs, including risk/long-run quotes</x:v>
+      </x:c>
+      <x:c r="E38" s="356" t="str">
+        <x:v>No-new-contract month close</x:v>
+      </x:c>
+      <x:c r="F38" s="356" t="str">
         <x:v>Recovery case costs</x:v>
       </x:c>
-      <x:c r="G38" s="268" t="str">
+      <x:c r="G38" s="356" t="str">
         <x:v>Recovery close before funding</x:v>
       </x:c>
-      <x:c r="H38" s="268" t="str">
+      <x:c r="H38" s="356" t="str">
         <x:v>Approved milestone release</x:v>
       </x:c>
-      <x:c r="I38" s="268" t="str">
+      <x:c r="I38" s="356" t="str">
         <x:v>Recovery close after funding</x:v>
       </x:c>
-      <x:c r="J38" s="268" t="str">
+      <x:c r="J38" s="356" t="str">
         <x:v>Change vs no-contract close</x:v>
       </x:c>
-      <x:c r="K38" s="265"/>
-      <x:c r="L38" s="265"/>
-      <x:c r="M38" s="265"/>
-      <x:c r="N38" s="265"/>
+      <x:c r="K38" s="353"/>
+      <x:c r="L38" s="353"/>
+      <x:c r="M38" s="353"/>
+      <x:c r="N38" s="353"/>
     </x:row>
     <x:row r="39" ht="28" customHeight="1">
       <x:c r="A39" s="165" t="str">
@@ -7282,23 +7604,23 @@
         <x:v>50000000</x:v>
       </x:c>
       <x:c r="C39" s="169" t="n">
-        <x:f>SUM('Economy'!$B$8:$B$9)</x:f>
+        <x:f>SUM('Economy'!$B$8:$B$9)+'Extended Cases'!$D$7+'Extended Cases'!$G$7+'Extended Cases'!$R$7</x:f>
         <x:v>5000000</x:v>
       </x:c>
       <x:c r="D39" s="169" t="n">
-        <x:f>SUM('Economy'!$B$10:$B$17)+'Economy'!$B$27</x:f>
+        <x:f>SUM('Economy'!$B$10:$B$18)+'Economy'!$B$27</x:f>
         <x:v>-1500000</x:v>
       </x:c>
       <x:c r="E39" s="177" t="n">
-        <x:f>B39+D39</x:f>
+        <x:f>B39+D39+'Extended Cases'!$D$7+'Extended Cases'!$G$7+'Extended Cases'!$P$7</x:f>
         <x:v>48500000</x:v>
       </x:c>
       <x:c r="F39" s="177" t="n">
-        <x:f>-(B28+D28)*'Economy'!$C$34*'Economy'!$C$32-'Economy'!$C$35*'Economy'!$C$32-(B28+D28)*'Economy'!$C$37*'Economy'!$C$32-D28*'Economy'!$C$45-E28*'Economy'!$C$51-F28*'Economy'!$C$53-G28*'Economy'!$C$47-H28*'Economy'!$C$49-C28*'Recovery &amp; Capital'!$C$7*'Economy'!$C$32-I28*'Recovery &amp; Capital'!$E$7-J28-K28-L28-M28</x:f>
+        <x:f>-(B28+D28)*'Economy'!$C$34*'Economy'!$C$32-'Economy'!$C$35*'Economy'!$C$32-(B28+D28)*'Economy'!$C$37*'Economy'!$C$32-D28*'Economy'!$C$45-E28*'Economy'!$C$51-F28*'Economy'!$C$53-G28*'Economy'!$C$47-H28*'Economy'!$C$49-C28*'Recovery &amp; Capital'!$C$7*'Economy'!$C$32-I28*'Recovery &amp; Capital'!$E$7-J28-K28-L28-M28-'Extended Cases'!$S$40</x:f>
         <x:v>-1500000</x:v>
       </x:c>
       <x:c r="G39" s="177" t="n">
-        <x:f>B39+F39</x:f>
+        <x:f>B39+F39+'Extended Cases'!$T$40</x:f>
         <x:v>48500000</x:v>
       </x:c>
       <x:c r="H39" s="177" t="n">
@@ -7327,7 +7649,7 @@
         <x:v>53500000</x:v>
       </x:c>
       <x:c r="C40" s="169" t="n">
-        <x:f>'Campaign Scenarios'!$C$44</x:f>
+        <x:f>'Campaign Scenarios'!$C$44+'Extended Cases'!$D$8+'Extended Cases'!$G$8+'Extended Cases'!$R$8</x:f>
         <x:v>5000000</x:v>
       </x:c>
       <x:c r="D40" s="169" t="n">
@@ -7335,15 +7657,15 @@
         <x:v>-2250000</x:v>
       </x:c>
       <x:c r="E40" s="177" t="n">
-        <x:f>B40+D40</x:f>
+        <x:f>B40+D40+'Extended Cases'!$D$8+'Extended Cases'!$G$8+'Extended Cases'!$P$8</x:f>
         <x:v>51250000</x:v>
       </x:c>
       <x:c r="F40" s="177" t="n">
-        <x:f>-(B29+D29)*'Campaign Scenarios'!$B$18*'Campaign Scenarios'!$C$32-'Campaign Scenarios'!$B$19*'Campaign Scenarios'!$C$32-(B29+D29)*'Campaign Scenarios'!$B$20*'Campaign Scenarios'!$C$32-D29*'Campaign Scenarios'!$B$21-E29*'Campaign Scenarios'!$B$22-F29*'Campaign Scenarios'!$B$23-G29*'Campaign Scenarios'!$B$24-H29*'Campaign Scenarios'!$B$25-C29*'Recovery &amp; Capital'!$C$8*'Campaign Scenarios'!$C$32-I29*'Recovery &amp; Capital'!$E$8-J29-K29-L29-M29</x:f>
+        <x:f>-(B29+D29)*'Campaign Scenarios'!$B$18*'Campaign Scenarios'!$C$32-'Campaign Scenarios'!$B$19*'Campaign Scenarios'!$C$32-(B29+D29)*'Campaign Scenarios'!$B$20*'Campaign Scenarios'!$C$32-D29*'Campaign Scenarios'!$B$21-E29*'Campaign Scenarios'!$B$22-F29*'Campaign Scenarios'!$B$23-G29*'Campaign Scenarios'!$B$24-H29*'Campaign Scenarios'!$B$25-C29*'Recovery &amp; Capital'!$C$8*'Campaign Scenarios'!$C$32-I29*'Recovery &amp; Capital'!$E$8-J29-K29-L29-M29-'Extended Cases'!$S$41</x:f>
         <x:v>-1500000</x:v>
       </x:c>
       <x:c r="G40" s="177" t="n">
-        <x:f>B40+F40</x:f>
+        <x:f>B40+F40+'Extended Cases'!$T$41</x:f>
         <x:v>52000000</x:v>
       </x:c>
       <x:c r="H40" s="177" t="n">
@@ -7372,7 +7694,7 @@
         <x:v>56250000</x:v>
       </x:c>
       <x:c r="C41" s="169" t="n">
-        <x:f>'Campaign Scenarios'!$C$74</x:f>
+        <x:f>'Campaign Scenarios'!$C$74+'Extended Cases'!$D$9+'Extended Cases'!$G$9+'Extended Cases'!$R$9</x:f>
         <x:v>30000000</x:v>
       </x:c>
       <x:c r="D41" s="169" t="n">
@@ -7380,15 +7702,15 @@
         <x:v>-4750000</x:v>
       </x:c>
       <x:c r="E41" s="177" t="n">
-        <x:f>B41+D41</x:f>
+        <x:f>B41+D41+'Extended Cases'!$D$9+'Extended Cases'!$G$9+'Extended Cases'!$P$9</x:f>
         <x:v>51500000</x:v>
       </x:c>
       <x:c r="F41" s="177" t="n">
-        <x:f>-(B30+D30)*'Campaign Scenarios'!$B$18*'Campaign Scenarios'!$C$62-'Campaign Scenarios'!$B$19*'Campaign Scenarios'!$C$62-(B30+D30)*'Campaign Scenarios'!$B$20*'Campaign Scenarios'!$C$62-D30*'Campaign Scenarios'!$B$21-E30*'Campaign Scenarios'!$B$22-F30*'Campaign Scenarios'!$B$23-G30*'Campaign Scenarios'!$B$24-H30*'Campaign Scenarios'!$B$25-C30*'Recovery &amp; Capital'!$C$9*'Campaign Scenarios'!$C$62-I30*'Recovery &amp; Capital'!$E$9-J30-K30-L30-M30</x:f>
+        <x:f>-(B30+D30)*'Campaign Scenarios'!$B$18*'Campaign Scenarios'!$C$62-'Campaign Scenarios'!$B$19*'Campaign Scenarios'!$C$62-(B30+D30)*'Campaign Scenarios'!$B$20*'Campaign Scenarios'!$C$62-D30*'Campaign Scenarios'!$B$21-E30*'Campaign Scenarios'!$B$22-F30*'Campaign Scenarios'!$B$23-G30*'Campaign Scenarios'!$B$24-H30*'Campaign Scenarios'!$B$25-C30*'Recovery &amp; Capital'!$C$9*'Campaign Scenarios'!$C$62-I30*'Recovery &amp; Capital'!$E$9-J30-K30-L30-M30-'Extended Cases'!$S$42</x:f>
         <x:v>-1500000</x:v>
       </x:c>
       <x:c r="G41" s="177" t="n">
-        <x:f>B41+F41</x:f>
+        <x:f>B41+F41+'Extended Cases'!$T$42</x:f>
         <x:v>54750000</x:v>
       </x:c>
       <x:c r="H41" s="177" t="n">
@@ -7417,7 +7739,7 @@
         <x:v>81500000</x:v>
       </x:c>
       <x:c r="C42" s="169" t="n">
-        <x:f>'Campaign Scenarios'!$C$104</x:f>
+        <x:f>'Campaign Scenarios'!$C$104+'Extended Cases'!$D$10+'Extended Cases'!$G$10+'Extended Cases'!$R$10</x:f>
         <x:v>100000000</x:v>
       </x:c>
       <x:c r="D42" s="169" t="n">
@@ -7425,15 +7747,15 @@
         <x:v>-12300000</x:v>
       </x:c>
       <x:c r="E42" s="177" t="n">
-        <x:f>B42+D42</x:f>
+        <x:f>B42+D42+'Extended Cases'!$D$10+'Extended Cases'!$G$10+'Extended Cases'!$P$10</x:f>
         <x:v>69200000</x:v>
       </x:c>
       <x:c r="F42" s="177" t="n">
-        <x:f>-(B31+D31)*'Campaign Scenarios'!$B$18*'Campaign Scenarios'!$C$92-'Campaign Scenarios'!$B$19*'Campaign Scenarios'!$C$92-(B31+D31)*'Campaign Scenarios'!$B$20*'Campaign Scenarios'!$C$92-D31*'Campaign Scenarios'!$B$21-E31*'Campaign Scenarios'!$B$22-F31*'Campaign Scenarios'!$B$23-G31*'Campaign Scenarios'!$B$24-H31*'Campaign Scenarios'!$B$25-C31*'Recovery &amp; Capital'!$C$10*'Campaign Scenarios'!$C$92-I31*'Recovery &amp; Capital'!$E$10-J31-K31-L31-M31</x:f>
+        <x:f>-(B31+D31)*'Campaign Scenarios'!$B$18*'Campaign Scenarios'!$C$92-'Campaign Scenarios'!$B$19*'Campaign Scenarios'!$C$92-(B31+D31)*'Campaign Scenarios'!$B$20*'Campaign Scenarios'!$C$92-D31*'Campaign Scenarios'!$B$21-E31*'Campaign Scenarios'!$B$22-F31*'Campaign Scenarios'!$B$23-G31*'Campaign Scenarios'!$B$24-H31*'Campaign Scenarios'!$B$25-C31*'Recovery &amp; Capital'!$C$10*'Campaign Scenarios'!$C$92-I31*'Recovery &amp; Capital'!$E$10-J31-K31-L31-M31-'Extended Cases'!$S$43</x:f>
         <x:v>-1800000</x:v>
       </x:c>
       <x:c r="G42" s="177" t="n">
-        <x:f>B42+F42</x:f>
+        <x:f>B42+F42+'Extended Cases'!$T$43</x:f>
         <x:v>79700000</x:v>
       </x:c>
       <x:c r="H42" s="177" t="n">
@@ -7462,7 +7784,7 @@
         <x:v>169200000</x:v>
       </x:c>
       <x:c r="C43" s="169" t="n">
-        <x:f>'Campaign Scenarios'!$C$134</x:f>
+        <x:f>'Campaign Scenarios'!$C$134+'Extended Cases'!$D$11+'Extended Cases'!$G$11+'Extended Cases'!$R$11</x:f>
         <x:v>375000000</x:v>
       </x:c>
       <x:c r="D43" s="169" t="n">
@@ -7470,15 +7792,15 @@
         <x:v>-25450000</x:v>
       </x:c>
       <x:c r="E43" s="177" t="n">
-        <x:f>B43+D43</x:f>
+        <x:f>B43+D43+'Extended Cases'!$D$11+'Extended Cases'!$G$11+'Extended Cases'!$P$11</x:f>
         <x:v>143750000</x:v>
       </x:c>
       <x:c r="F43" s="177" t="n">
-        <x:f>-(B32+D32)*'Campaign Scenarios'!$B$18*'Campaign Scenarios'!$C$122-'Campaign Scenarios'!$B$19*'Campaign Scenarios'!$C$122-(B32+D32)*'Campaign Scenarios'!$B$20*'Campaign Scenarios'!$C$122-D32*'Campaign Scenarios'!$B$21-E32*'Campaign Scenarios'!$B$22-F32*'Campaign Scenarios'!$B$23-G32*'Campaign Scenarios'!$B$24-H32*'Campaign Scenarios'!$B$25-C32*'Recovery &amp; Capital'!$C$11*'Campaign Scenarios'!$C$122-I32*'Recovery &amp; Capital'!$E$11-J32-K32-L32-M32</x:f>
+        <x:f>-(B32+D32)*'Campaign Scenarios'!$B$18*'Campaign Scenarios'!$C$122-'Campaign Scenarios'!$B$19*'Campaign Scenarios'!$C$122-(B32+D32)*'Campaign Scenarios'!$B$20*'Campaign Scenarios'!$C$122-D32*'Campaign Scenarios'!$B$21-E32*'Campaign Scenarios'!$B$22-F32*'Campaign Scenarios'!$B$23-G32*'Campaign Scenarios'!$B$24-H32*'Campaign Scenarios'!$B$25-C32*'Recovery &amp; Capital'!$C$11*'Campaign Scenarios'!$C$122-I32*'Recovery &amp; Capital'!$E$11-J32-K32-L32-M32-'Extended Cases'!$S$44</x:f>
         <x:v>-1950000</x:v>
       </x:c>
       <x:c r="G43" s="177" t="n">
-        <x:f>B43+F43</x:f>
+        <x:f>B43+F43+'Extended Cases'!$T$44</x:f>
         <x:v>167250000</x:v>
       </x:c>
       <x:c r="H43" s="177" t="n">
@@ -7507,7 +7829,7 @@
         <x:v>518750000</x:v>
       </x:c>
       <x:c r="C44" s="169" t="n">
-        <x:f>'Campaign Scenarios'!$C$164</x:f>
+        <x:f>'Campaign Scenarios'!$C$164+'Extended Cases'!$D$12+'Extended Cases'!$G$12+'Extended Cases'!$R$12</x:f>
         <x:v>750000000</x:v>
       </x:c>
       <x:c r="D44" s="169" t="n">
@@ -7515,15 +7837,15 @@
         <x:v>-65250000</x:v>
       </x:c>
       <x:c r="E44" s="177" t="n">
-        <x:f>B44+D44</x:f>
+        <x:f>B44+D44+'Extended Cases'!$D$12+'Extended Cases'!$G$12+'Extended Cases'!$P$12</x:f>
         <x:v>453500000</x:v>
       </x:c>
       <x:c r="F44" s="177" t="n">
-        <x:f>-(B33+D33)*'Campaign Scenarios'!$B$18*'Campaign Scenarios'!$C$152-'Campaign Scenarios'!$B$19*'Campaign Scenarios'!$C$152-(B33+D33)*'Campaign Scenarios'!$B$20*'Campaign Scenarios'!$C$152-D33*'Campaign Scenarios'!$B$21-E33*'Campaign Scenarios'!$B$22-F33*'Campaign Scenarios'!$B$23-G33*'Campaign Scenarios'!$B$24-H33*'Campaign Scenarios'!$B$25-C33*'Recovery &amp; Capital'!$C$12*'Campaign Scenarios'!$C$152-I33*'Recovery &amp; Capital'!$E$12-J33-K33-L33-M33</x:f>
+        <x:f>-(B33+D33)*'Campaign Scenarios'!$B$18*'Campaign Scenarios'!$C$152-'Campaign Scenarios'!$B$19*'Campaign Scenarios'!$C$152-(B33+D33)*'Campaign Scenarios'!$B$20*'Campaign Scenarios'!$C$152-D33*'Campaign Scenarios'!$B$21-E33*'Campaign Scenarios'!$B$22-F33*'Campaign Scenarios'!$B$23-G33*'Campaign Scenarios'!$B$24-H33*'Campaign Scenarios'!$B$25-C33*'Recovery &amp; Capital'!$C$12*'Campaign Scenarios'!$C$152-I33*'Recovery &amp; Capital'!$E$12-J33-K33-L33-M33-'Extended Cases'!$S$45</x:f>
         <x:v>-2250000</x:v>
       </x:c>
       <x:c r="G44" s="177" t="n">
-        <x:f>B44+F44</x:f>
+        <x:f>B44+F44+'Extended Cases'!$T$45</x:f>
         <x:v>516500000</x:v>
       </x:c>
       <x:c r="H44" s="177" t="n">
@@ -7552,7 +7874,7 @@
         <x:v>1203500000</x:v>
       </x:c>
       <x:c r="C45" s="169" t="n">
-        <x:f>'Campaign Scenarios'!$C$194</x:f>
+        <x:f>'Campaign Scenarios'!$C$194+'Extended Cases'!$D$13+'Extended Cases'!$G$13+'Extended Cases'!$R$13</x:f>
         <x:v>1200000000</x:v>
       </x:c>
       <x:c r="D45" s="169" t="n">
@@ -7560,15 +7882,15 @@
         <x:v>-118500000</x:v>
       </x:c>
       <x:c r="E45" s="177" t="n">
-        <x:f>B45+D45</x:f>
+        <x:f>B45+D45+'Extended Cases'!$D$13+'Extended Cases'!$G$13+'Extended Cases'!$P$13</x:f>
         <x:v>1085000000</x:v>
       </x:c>
       <x:c r="F45" s="177" t="n">
-        <x:f>-(B34+D34)*'Campaign Scenarios'!$B$18*'Campaign Scenarios'!$C$182-'Campaign Scenarios'!$B$19*'Campaign Scenarios'!$C$182-(B34+D34)*'Campaign Scenarios'!$B$20*'Campaign Scenarios'!$C$182-D34*'Campaign Scenarios'!$B$21-E34*'Campaign Scenarios'!$B$22-F34*'Campaign Scenarios'!$B$23-G34*'Campaign Scenarios'!$B$24-H34*'Campaign Scenarios'!$B$25-C34*'Recovery &amp; Capital'!$C$13*'Campaign Scenarios'!$C$182-I34*'Recovery &amp; Capital'!$E$13-J34-K34-L34-M34</x:f>
+        <x:f>-(B34+D34)*'Campaign Scenarios'!$B$18*'Campaign Scenarios'!$C$182-'Campaign Scenarios'!$B$19*'Campaign Scenarios'!$C$182-(B34+D34)*'Campaign Scenarios'!$B$20*'Campaign Scenarios'!$C$182-D34*'Campaign Scenarios'!$B$21-E34*'Campaign Scenarios'!$B$22-F34*'Campaign Scenarios'!$B$23-G34*'Campaign Scenarios'!$B$24-H34*'Campaign Scenarios'!$B$25-C34*'Recovery &amp; Capital'!$C$13*'Campaign Scenarios'!$C$182-I34*'Recovery &amp; Capital'!$E$13-J34-K34-L34-M34-'Extended Cases'!$S$46</x:f>
         <x:v>-2250000</x:v>
       </x:c>
       <x:c r="G45" s="177" t="n">
-        <x:f>B45+F45</x:f>
+        <x:f>B45+F45+'Extended Cases'!$T$46</x:f>
         <x:v>1201250000</x:v>
       </x:c>
       <x:c r="H45" s="177" t="n">
@@ -7644,4 +7966,2269 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="19" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="17" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="20" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="21" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="38" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="36" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="18" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="23" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="23" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="24" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="22" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="48" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="21" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="50" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="10"/>
+      <x:c r="B1" s="10"/>
+      <x:c r="C1" s="10"/>
+      <x:c r="D1" s="10"/>
+      <x:c r="E1" s="10"/>
+      <x:c r="F1" s="10"/>
+      <x:c r="G1" s="10"/>
+      <x:c r="H1" s="10"/>
+      <x:c r="I1" s="10"/>
+      <x:c r="J1" s="10"/>
+      <x:c r="K1" s="10"/>
+      <x:c r="L1" s="10"/>
+      <x:c r="M1" s="10"/>
+      <x:c r="N1" s="10"/>
+      <x:c r="O1" s="10"/>
+      <x:c r="P1" s="10"/>
+      <x:c r="Q1" s="10"/>
+      <x:c r="R1" s="10"/>
+      <x:c r="S1" s="10"/>
+      <x:c r="T1" s="10"/>
+      <x:c r="U1" s="10"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="163" t="str">
+        <x:v>Rimrooms - Async Industries: extended economy cases</x:v>
+      </x:c>
+      <x:c r="B2" s="10"/>
+      <x:c r="C2" s="10"/>
+      <x:c r="D2" s="10"/>
+      <x:c r="E2" s="10"/>
+      <x:c r="F2" s="10"/>
+      <x:c r="G2" s="10"/>
+      <x:c r="H2" s="10"/>
+      <x:c r="I2" s="10"/>
+      <x:c r="J2" s="10"/>
+      <x:c r="K2" s="10"/>
+      <x:c r="L2" s="10"/>
+      <x:c r="M2" s="10"/>
+      <x:c r="N2" s="10"/>
+      <x:c r="O2" s="10"/>
+      <x:c r="P2" s="10"/>
+      <x:c r="Q2" s="10"/>
+      <x:c r="R2" s="10"/>
+      <x:c r="S2" s="10"/>
+      <x:c r="T2" s="10"/>
+      <x:c r="U2" s="10"/>
+    </x:row>
+    <x:row r="3" ht="22" customHeight="1">
+      <x:c r="A3" s="251" t="str">
+        <x:v>Editable pre-code hypotheses, default zero. Only accepted/delivered work, earned leases, signed penalties, and approved claims post; goods and vehicles remain physical inventory.</x:v>
+      </x:c>
+      <x:c r="B3" s="251"/>
+      <x:c r="C3" s="251"/>
+      <x:c r="D3" s="251"/>
+      <x:c r="E3" s="251"/>
+      <x:c r="F3" s="251"/>
+      <x:c r="G3" s="251"/>
+      <x:c r="H3" s="251"/>
+      <x:c r="I3" s="251"/>
+      <x:c r="J3" s="251"/>
+      <x:c r="K3" s="251"/>
+      <x:c r="L3" s="251"/>
+      <x:c r="M3" s="251"/>
+      <x:c r="N3" s="251"/>
+      <x:c r="O3" s="251"/>
+      <x:c r="P3" s="251"/>
+      <x:c r="Q3" s="251"/>
+      <x:c r="R3" s="251"/>
+      <x:c r="S3" s="251"/>
+      <x:c r="T3" s="10"/>
+      <x:c r="U3" s="10"/>
+    </x:row>
+    <x:row r="4" ht="24" customHeight="1">
+      <x:c r="A4" s="251" t="str">
+        <x:v>Optional VGE costs are scenarios, not a dependency. Expedition extension costs are added beyond the monthly base horizon. Enter only incremental amounts; do not double-count costs already entered on the other workbook sheets.</x:v>
+      </x:c>
+      <x:c r="B4" s="251"/>
+      <x:c r="C4" s="251"/>
+      <x:c r="D4" s="251"/>
+      <x:c r="E4" s="251"/>
+      <x:c r="F4" s="251"/>
+      <x:c r="G4" s="251"/>
+      <x:c r="H4" s="251"/>
+      <x:c r="I4" s="251"/>
+      <x:c r="J4" s="251"/>
+      <x:c r="K4" s="251"/>
+      <x:c r="L4" s="251"/>
+      <x:c r="M4" s="251"/>
+      <x:c r="N4" s="251"/>
+      <x:c r="O4" s="251"/>
+      <x:c r="P4" s="251"/>
+      <x:c r="Q4" s="251"/>
+      <x:c r="R4" s="251"/>
+      <x:c r="S4" s="251"/>
+      <x:c r="T4" s="10"/>
+      <x:c r="U4" s="10"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="351" t="str">
+        <x:v>Separate receipts, capped penalties, and cargo incidents</x:v>
+      </x:c>
+      <x:c r="B5" s="351"/>
+      <x:c r="C5" s="351"/>
+      <x:c r="D5" s="351"/>
+      <x:c r="E5" s="351"/>
+      <x:c r="F5" s="351"/>
+      <x:c r="G5" s="351"/>
+      <x:c r="H5" s="351"/>
+      <x:c r="I5" s="351"/>
+      <x:c r="J5" s="351"/>
+      <x:c r="K5" s="351"/>
+      <x:c r="L5" s="351"/>
+      <x:c r="M5" s="351"/>
+      <x:c r="N5" s="351"/>
+      <x:c r="O5" s="351"/>
+      <x:c r="P5" s="351"/>
+      <x:c r="Q5" s="351"/>
+      <x:c r="R5" s="351"/>
+      <x:c r="S5" s="351"/>
+      <x:c r="T5" s="10"/>
+      <x:c r="U5" s="10"/>
+    </x:row>
+    <x:row r="6" ht="62" customHeight="1">
+      <x:c r="A6" s="353" t="str">
+        <x:v>Campaign stage</x:v>
+      </x:c>
+      <x:c r="B6" s="353" t="str">
+        <x:v>Separate service deliveries / month</x:v>
+      </x:c>
+      <x:c r="C6" s="353" t="str">
+        <x:v>Receipt per accepted service (USD)</x:v>
+      </x:c>
+      <x:c r="D6" s="353" t="str">
+        <x:v>Service receipts (USD)</x:v>
+      </x:c>
+      <x:c r="E6" s="353" t="str">
+        <x:v>Billable lease days</x:v>
+      </x:c>
+      <x:c r="F6" s="353" t="str">
+        <x:v>Receipt per earned day (USD)</x:v>
+      </x:c>
+      <x:c r="G6" s="353" t="str">
+        <x:v>Lease receipts (USD)</x:v>
+      </x:c>
+      <x:c r="H6" s="353" t="str">
+        <x:v>Contracts with penalty due</x:v>
+      </x:c>
+      <x:c r="I6" s="353" t="str">
+        <x:v>Claimed penalty per contract (USD)</x:v>
+      </x:c>
+      <x:c r="J6" s="353" t="str">
+        <x:v>Average accepted contract value cap basis (USD)</x:v>
+      </x:c>
+      <x:c r="K6" s="353" t="str">
+        <x:v>Penalty after 25% cap (USD)</x:v>
+      </x:c>
+      <x:c r="L6" s="353" t="str">
+        <x:v>Cargo/crew incident count</x:v>
+      </x:c>
+      <x:c r="M6" s="353" t="str">
+        <x:v>Response/rescue per incident (USD)</x:v>
+      </x:c>
+      <x:c r="N6" s="353" t="str">
+        <x:v>Incident response cost (USD)</x:v>
+      </x:c>
+      <x:c r="O6" s="353" t="str">
+        <x:v>Contract receipts delayed/lost this period (USD)</x:v>
+      </x:c>
+      <x:c r="P6" s="353" t="str">
+        <x:v>Accepted claim reimbursement received (USD)</x:v>
+      </x:c>
+      <x:c r="Q6" s="353" t="str">
+        <x:v>Core contract receipts before incident adjustment (USD)</x:v>
+      </x:c>
+      <x:c r="R6" s="353" t="str">
+        <x:v>Incident receipt adjustment (USD)</x:v>
+      </x:c>
+      <x:c r="S6" s="353" t="str">
+        <x:v>Basis / status</x:v>
+      </x:c>
+      <x:c r="T6" s="10"/>
+      <x:c r="U6" s="10"/>
+    </x:row>
+    <x:row r="7" ht="60" customHeight="1">
+      <x:c r="A7" s="313" t="str">
+        <x:v>Stage 1: First safe survey</x:v>
+      </x:c>
+      <x:c r="B7" s="365" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C7" s="366" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D7" s="300" t="n">
+        <x:f>B7*C7</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E7" s="365" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F7" s="366" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G7" s="300" t="n">
+        <x:f>E7*F7</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H7" s="371" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I7" s="372" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J7" s="310" t="n">
+        <x:f>'Economy'!$C$39</x:f>
+        <x:v>5000000</x:v>
+      </x:c>
+      <x:c r="K7" s="310" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L7" s="365" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M7" s="366" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N7" s="300" t="n">
+        <x:f>MAX(0,L7)*MAX(0,M7)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O7" s="366" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P7" s="366" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q7" s="310" t="n">
+        <x:f>SUM('Economy'!$B$8:$B$9)</x:f>
+        <x:v>5000000</x:v>
+      </x:c>
+      <x:c r="R7" s="310" t="n">
+        <x:f>MAX(0,P7)-MIN(MAX(0,O7),MAX(0,Q7))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S7" s="301" t="str">
+        <x:v>Stage 1 penalties remain in Economy.</x:v>
+      </x:c>
+      <x:c r="T7" s="10"/>
+      <x:c r="U7" s="10"/>
+    </x:row>
+    <x:row r="8" ht="60" customHeight="1">
+      <x:c r="A8" s="165" t="str">
+        <x:v>Stage 2: Repeat access</x:v>
+      </x:c>
+      <x:c r="B8" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C8" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D8" s="304" t="n">
+        <x:f>B8*C8</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E8" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F8" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G8" s="304" t="n">
+        <x:f>E8*F8</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H8" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I8" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J8" s="169" t="n">
+        <x:f>'Campaign Scenarios'!$C$37</x:f>
+        <x:v>2500000</x:v>
+      </x:c>
+      <x:c r="K8" s="169" t="n">
+        <x:f>MAX(0,H8)*MIN(MAX(0,I8),MAX(0,J8)*25%)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L8" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M8" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N8" s="304" t="n">
+        <x:f>MAX(0,L8)*MAX(0,M8)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O8" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P8" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q8" s="169" t="n">
+        <x:f>'Campaign Scenarios'!$C$44</x:f>
+        <x:v>5000000</x:v>
+      </x:c>
+      <x:c r="R8" s="169" t="n">
+        <x:f>MAX(0,P8)-MIN(MAX(0,O8),MAX(0,Q8))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S8" s="170" t="str">
+        <x:v>Count accepted work/claims only; delayed cash is held.</x:v>
+      </x:c>
+      <x:c r="T8" s="10"/>
+      <x:c r="U8" s="10"/>
+    </x:row>
+    <x:row r="9" ht="60" customHeight="1">
+      <x:c r="A9" s="165" t="str">
+        <x:v>Stage 3: Specialist services</x:v>
+      </x:c>
+      <x:c r="B9" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C9" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D9" s="304" t="n">
+        <x:f>B9*C9</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E9" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F9" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G9" s="304" t="n">
+        <x:f>E9*F9</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H9" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I9" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J9" s="169" t="n">
+        <x:f>'Campaign Scenarios'!$C$67</x:f>
+        <x:v>10000000</x:v>
+      </x:c>
+      <x:c r="K9" s="169" t="n">
+        <x:f>MAX(0,H9)*MIN(MAX(0,I9),MAX(0,J9)*25%)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L9" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M9" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N9" s="304" t="n">
+        <x:f>MAX(0,L9)*MAX(0,M9)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O9" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P9" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q9" s="169" t="n">
+        <x:f>'Campaign Scenarios'!$C$74</x:f>
+        <x:v>30000000</x:v>
+      </x:c>
+      <x:c r="R9" s="169" t="n">
+        <x:f>MAX(0,P9)-MIN(MAX(0,O9),MAX(0,Q9))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S9" s="170" t="str">
+        <x:v>Count accepted work/claims only; delayed cash is held.</x:v>
+      </x:c>
+      <x:c r="T9" s="10"/>
+      <x:c r="U9" s="10"/>
+    </x:row>
+    <x:row r="10" ht="60" customHeight="1">
+      <x:c r="A10" s="165" t="str">
+        <x:v>Stage 4: Leases and remote sites</x:v>
+      </x:c>
+      <x:c r="B10" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C10" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D10" s="304" t="n">
+        <x:f>B10*C10</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E10" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F10" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G10" s="304" t="n">
+        <x:f>E10*F10</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H10" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I10" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J10" s="169" t="n">
+        <x:f>'Campaign Scenarios'!$C$97</x:f>
+        <x:v>25000000</x:v>
+      </x:c>
+      <x:c r="K10" s="169" t="n">
+        <x:f>MAX(0,H10)*MIN(MAX(0,I10),MAX(0,J10)*25%)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L10" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M10" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N10" s="304" t="n">
+        <x:f>MAX(0,L10)*MAX(0,M10)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O10" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P10" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q10" s="169" t="n">
+        <x:f>'Campaign Scenarios'!$C$104</x:f>
+        <x:v>100000000</x:v>
+      </x:c>
+      <x:c r="R10" s="169" t="n">
+        <x:f>MAX(0,P10)-MIN(MAX(0,O10),MAX(0,Q10))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S10" s="170" t="str">
+        <x:v>Count accepted work/claims only; delayed cash is held.</x:v>
+      </x:c>
+      <x:c r="T10" s="10"/>
+      <x:c r="U10" s="10"/>
+    </x:row>
+    <x:row r="11" ht="60" customHeight="1">
+      <x:c r="A11" s="165" t="str">
+        <x:v>Stage 5: Large recovery and network work</x:v>
+      </x:c>
+      <x:c r="B11" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C11" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D11" s="304" t="n">
+        <x:f>B11*C11</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E11" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F11" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G11" s="304" t="n">
+        <x:f>E11*F11</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H11" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I11" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J11" s="169" t="n">
+        <x:f>'Campaign Scenarios'!$C$127</x:f>
+        <x:v>75000000</x:v>
+      </x:c>
+      <x:c r="K11" s="169" t="n">
+        <x:f>MAX(0,H11)*MIN(MAX(0,I11),MAX(0,J11)*25%)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L11" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M11" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N11" s="304" t="n">
+        <x:f>MAX(0,L11)*MAX(0,M11)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O11" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P11" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q11" s="169" t="n">
+        <x:f>'Campaign Scenarios'!$C$134</x:f>
+        <x:v>375000000</x:v>
+      </x:c>
+      <x:c r="R11" s="169" t="n">
+        <x:f>MAX(0,P11)-MIN(MAX(0,O11),MAX(0,Q11))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S11" s="170" t="str">
+        <x:v>Count accepted work/claims only; delayed cash is held.</x:v>
+      </x:c>
+      <x:c r="T11" s="10"/>
+      <x:c r="U11" s="10"/>
+    </x:row>
+    <x:row r="12" ht="60" customHeight="1">
+      <x:c r="A12" s="165" t="str">
+        <x:v>Stage 6: Vehicle and optional orbital support</x:v>
+      </x:c>
+      <x:c r="B12" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C12" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D12" s="304" t="n">
+        <x:f>B12*C12</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E12" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F12" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G12" s="304" t="n">
+        <x:f>E12*F12</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H12" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I12" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J12" s="169" t="n">
+        <x:f>'Campaign Scenarios'!$C$157</x:f>
+        <x:v>150000000</x:v>
+      </x:c>
+      <x:c r="K12" s="169" t="n">
+        <x:f>MAX(0,H12)*MIN(MAX(0,I12),MAX(0,J12)*25%)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L12" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M12" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N12" s="304" t="n">
+        <x:f>MAX(0,L12)*MAX(0,M12)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O12" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P12" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q12" s="169" t="n">
+        <x:f>'Campaign Scenarios'!$C$164</x:f>
+        <x:v>750000000</x:v>
+      </x:c>
+      <x:c r="R12" s="169" t="n">
+        <x:f>MAX(0,P12)-MIN(MAX(0,O12),MAX(0,Q12))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S12" s="170" t="str">
+        <x:v>Count accepted work/claims only; delayed cash is held.</x:v>
+      </x:c>
+      <x:c r="T12" s="10"/>
+      <x:c r="U12" s="10"/>
+    </x:row>
+    <x:row r="13" ht="60" customHeight="1">
+      <x:c r="A13" s="165" t="str">
+        <x:v>Stage 7: Deep-site operations</x:v>
+      </x:c>
+      <x:c r="B13" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C13" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D13" s="304" t="n">
+        <x:f>B13*C13</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E13" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F13" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G13" s="304" t="n">
+        <x:f>E13*F13</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H13" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I13" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J13" s="169" t="n">
+        <x:f>'Campaign Scenarios'!$C$187</x:f>
+        <x:v>300000000</x:v>
+      </x:c>
+      <x:c r="K13" s="169" t="n">
+        <x:f>MAX(0,H13)*MIN(MAX(0,I13),MAX(0,J13)*25%)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L13" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M13" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N13" s="304" t="n">
+        <x:f>MAX(0,L13)*MAX(0,M13)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O13" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P13" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q13" s="169" t="n">
+        <x:f>'Campaign Scenarios'!$C$194</x:f>
+        <x:v>1200000000</x:v>
+      </x:c>
+      <x:c r="R13" s="169" t="n">
+        <x:f>MAX(0,P13)-MIN(MAX(0,O13),MAX(0,Q13))</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S13" s="170" t="str">
+        <x:v>Count accepted work/claims only; delayed cash is held.</x:v>
+      </x:c>
+      <x:c r="T13" s="10"/>
+      <x:c r="U13" s="10"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="10"/>
+      <x:c r="B14" s="10"/>
+      <x:c r="C14" s="10"/>
+      <x:c r="D14" s="10"/>
+      <x:c r="E14" s="10"/>
+      <x:c r="F14" s="10"/>
+      <x:c r="G14" s="10"/>
+      <x:c r="H14" s="10"/>
+      <x:c r="I14" s="10"/>
+      <x:c r="J14" s="10"/>
+      <x:c r="K14" s="10"/>
+      <x:c r="L14" s="10"/>
+      <x:c r="M14" s="10"/>
+      <x:c r="N14" s="10"/>
+      <x:c r="O14" s="10"/>
+      <x:c r="P14" s="10"/>
+      <x:c r="Q14" s="10"/>
+      <x:c r="R14" s="10"/>
+      <x:c r="S14" s="10"/>
+      <x:c r="T14" s="10"/>
+      <x:c r="U14" s="10"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="10"/>
+      <x:c r="B15" s="10"/>
+      <x:c r="C15" s="10"/>
+      <x:c r="D15" s="10"/>
+      <x:c r="E15" s="10"/>
+      <x:c r="F15" s="10"/>
+      <x:c r="G15" s="10"/>
+      <x:c r="H15" s="10"/>
+      <x:c r="I15" s="10"/>
+      <x:c r="J15" s="10"/>
+      <x:c r="K15" s="10"/>
+      <x:c r="L15" s="10"/>
+      <x:c r="M15" s="10"/>
+      <x:c r="N15" s="10"/>
+      <x:c r="O15" s="10"/>
+      <x:c r="P15" s="10"/>
+      <x:c r="Q15" s="10"/>
+      <x:c r="R15" s="10"/>
+      <x:c r="S15" s="10"/>
+      <x:c r="T15" s="10"/>
+      <x:c r="U15" s="10"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="351" t="str">
+        <x:v>Optional VGE vehicle/gravship and itemized outpost case</x:v>
+      </x:c>
+      <x:c r="B16" s="351"/>
+      <x:c r="C16" s="351"/>
+      <x:c r="D16" s="351"/>
+      <x:c r="E16" s="351"/>
+      <x:c r="F16" s="351"/>
+      <x:c r="G16" s="351"/>
+      <x:c r="H16" s="351"/>
+      <x:c r="I16" s="351"/>
+      <x:c r="J16" s="351"/>
+      <x:c r="K16" s="351"/>
+      <x:c r="L16" s="351"/>
+      <x:c r="M16" s="10"/>
+      <x:c r="N16" s="10"/>
+      <x:c r="O16" s="10"/>
+      <x:c r="P16" s="10"/>
+      <x:c r="Q16" s="10"/>
+      <x:c r="R16" s="10"/>
+      <x:c r="S16" s="10"/>
+      <x:c r="T16" s="10"/>
+      <x:c r="U16" s="10"/>
+    </x:row>
+    <x:row r="17" ht="64" customHeight="1">
+      <x:c r="A17" s="353" t="str">
+        <x:v>Campaign stage</x:v>
+      </x:c>
+      <x:c r="B17" s="353" t="str">
+        <x:v>Optional vehicle/gravship acquisition quote (USD)</x:v>
+      </x:c>
+      <x:c r="C17" s="353" t="str">
+        <x:v>Vehicle/gravship operating, fuel, maintenance quote (USD / case)</x:v>
+      </x:c>
+      <x:c r="D17" s="353" t="str">
+        <x:v>Additional outpost hires beyond stage roster (FTE)</x:v>
+      </x:c>
+      <x:c r="E17" s="353" t="str">
+        <x:v>Outpost extra payroll + setup (USD)</x:v>
+      </x:c>
+      <x:c r="F17" s="353" t="str">
+        <x:v>Outpost security/defense quote (USD)</x:v>
+      </x:c>
+      <x:c r="G17" s="353" t="str">
+        <x:v>Physical resupply shipments (count)</x:v>
+      </x:c>
+      <x:c r="H17" s="353" t="str">
+        <x:v>Invoice per physical shipment (USD)</x:v>
+      </x:c>
+      <x:c r="I17" s="353" t="str">
+        <x:v>Extra communications beyond basic site allowance (USD)</x:v>
+      </x:c>
+      <x:c r="J17" s="353" t="str">
+        <x:v>Evacuation/closure reserve quote (USD)</x:v>
+      </x:c>
+      <x:c r="K17" s="353" t="str">
+        <x:v>Total vehicle + outpost additions (USD)</x:v>
+      </x:c>
+      <x:c r="L17" s="353" t="str">
+        <x:v>Basis / status</x:v>
+      </x:c>
+      <x:c r="M17" s="10"/>
+      <x:c r="N17" s="10"/>
+      <x:c r="O17" s="10"/>
+      <x:c r="P17" s="10"/>
+      <x:c r="Q17" s="10"/>
+      <x:c r="R17" s="10"/>
+      <x:c r="S17" s="10"/>
+      <x:c r="T17" s="10"/>
+      <x:c r="U17" s="10"/>
+    </x:row>
+    <x:row r="18" ht="60" customHeight="1">
+      <x:c r="A18" s="313" t="str">
+        <x:v>Stage 1: First safe survey</x:v>
+      </x:c>
+      <x:c r="B18" s="366" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C18" s="366" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D18" s="365" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E18" s="310" t="n">
+        <x:f>MAX(0,D18)*(30*'Economy'!$C$34+'Economy'!$C$45)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F18" s="366" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G18" s="365" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H18" s="366" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I18" s="366" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J18" s="366" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K18" s="310" t="n">
+        <x:f>SUM(B18:C18)+E18+F18+G18*H18+I18+J18</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L18" s="301" t="str">
+        <x:v>VGE is optional; delivered vehicles stay physical. Base site fee is included.</x:v>
+      </x:c>
+      <x:c r="M18" s="10"/>
+      <x:c r="N18" s="10"/>
+      <x:c r="O18" s="10"/>
+      <x:c r="P18" s="10"/>
+      <x:c r="Q18" s="10"/>
+      <x:c r="R18" s="10"/>
+      <x:c r="S18" s="10"/>
+      <x:c r="T18" s="10"/>
+      <x:c r="U18" s="10"/>
+    </x:row>
+    <x:row r="19" ht="60" customHeight="1">
+      <x:c r="A19" s="165" t="str">
+        <x:v>Stage 2: Repeat access</x:v>
+      </x:c>
+      <x:c r="B19" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C19" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D19" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E19" s="169" t="n">
+        <x:f>MAX(0,D19)*(30*'Campaign Scenarios'!$B$18+'Campaign Scenarios'!$B$21)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F19" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G19" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H19" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I19" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J19" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K19" s="169" t="n">
+        <x:f>SUM(B19:C19)+E19+F19+G19*H19+I19+J19</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L19" s="170" t="str">
+        <x:v>VGE is optional; delivered vehicles stay physical. Base site fee is included.</x:v>
+      </x:c>
+      <x:c r="M19" s="10"/>
+      <x:c r="N19" s="10"/>
+      <x:c r="O19" s="10"/>
+      <x:c r="P19" s="10"/>
+      <x:c r="Q19" s="10"/>
+      <x:c r="R19" s="10"/>
+      <x:c r="S19" s="10"/>
+      <x:c r="T19" s="10"/>
+      <x:c r="U19" s="10"/>
+    </x:row>
+    <x:row r="20" ht="60" customHeight="1">
+      <x:c r="A20" s="165" t="str">
+        <x:v>Stage 3: Specialist services</x:v>
+      </x:c>
+      <x:c r="B20" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C20" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D20" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E20" s="169" t="n">
+        <x:f>MAX(0,D20)*(30*'Campaign Scenarios'!$B$18+'Campaign Scenarios'!$B$21)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F20" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G20" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H20" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I20" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J20" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K20" s="169" t="n">
+        <x:f>SUM(B20:C20)+E20+F20+G20*H20+I20+J20</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L20" s="170" t="str">
+        <x:v>VGE is optional; delivered vehicles stay physical. Base site fee is included.</x:v>
+      </x:c>
+      <x:c r="M20" s="10"/>
+      <x:c r="N20" s="10"/>
+      <x:c r="O20" s="10"/>
+      <x:c r="P20" s="10"/>
+      <x:c r="Q20" s="10"/>
+      <x:c r="R20" s="10"/>
+      <x:c r="S20" s="10"/>
+      <x:c r="T20" s="10"/>
+      <x:c r="U20" s="10"/>
+    </x:row>
+    <x:row r="21" ht="60" customHeight="1">
+      <x:c r="A21" s="165" t="str">
+        <x:v>Stage 4: Leases and remote sites</x:v>
+      </x:c>
+      <x:c r="B21" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C21" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D21" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E21" s="169" t="n">
+        <x:f>MAX(0,D21)*(30*'Campaign Scenarios'!$B$18+'Campaign Scenarios'!$B$21)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F21" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G21" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H21" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I21" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J21" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K21" s="169" t="n">
+        <x:f>SUM(B21:C21)+E21+F21+G21*H21+I21+J21</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L21" s="170" t="str">
+        <x:v>VGE is optional; delivered vehicles stay physical. Base site fee is included.</x:v>
+      </x:c>
+      <x:c r="M21" s="10"/>
+      <x:c r="N21" s="10"/>
+      <x:c r="O21" s="10"/>
+      <x:c r="P21" s="10"/>
+      <x:c r="Q21" s="10"/>
+      <x:c r="R21" s="10"/>
+      <x:c r="S21" s="10"/>
+      <x:c r="T21" s="10"/>
+      <x:c r="U21" s="10"/>
+    </x:row>
+    <x:row r="22" ht="60" customHeight="1">
+      <x:c r="A22" s="165" t="str">
+        <x:v>Stage 5: Large recovery and network work</x:v>
+      </x:c>
+      <x:c r="B22" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C22" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D22" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E22" s="169" t="n">
+        <x:f>MAX(0,D22)*(30*'Campaign Scenarios'!$B$18+'Campaign Scenarios'!$B$21)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F22" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G22" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H22" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I22" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J22" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K22" s="169" t="n">
+        <x:f>SUM(B22:C22)+E22+F22+G22*H22+I22+J22</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L22" s="170" t="str">
+        <x:v>VGE is optional; delivered vehicles stay physical. Base site fee is included.</x:v>
+      </x:c>
+      <x:c r="M22" s="10"/>
+      <x:c r="N22" s="10"/>
+      <x:c r="O22" s="10"/>
+      <x:c r="P22" s="10"/>
+      <x:c r="Q22" s="10"/>
+      <x:c r="R22" s="10"/>
+      <x:c r="S22" s="10"/>
+      <x:c r="T22" s="10"/>
+      <x:c r="U22" s="10"/>
+    </x:row>
+    <x:row r="23" ht="60" customHeight="1">
+      <x:c r="A23" s="165" t="str">
+        <x:v>Stage 6: Vehicle and optional orbital support</x:v>
+      </x:c>
+      <x:c r="B23" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C23" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D23" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E23" s="169" t="n">
+        <x:f>MAX(0,D23)*(30*'Campaign Scenarios'!$B$18+'Campaign Scenarios'!$B$21)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F23" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G23" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H23" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I23" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J23" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K23" s="169" t="n">
+        <x:f>SUM(B23:C23)+E23+F23+G23*H23+I23+J23</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L23" s="170" t="str">
+        <x:v>VGE is optional; delivered vehicles stay physical. Base site fee is included.</x:v>
+      </x:c>
+      <x:c r="M23" s="10"/>
+      <x:c r="N23" s="10"/>
+      <x:c r="O23" s="10"/>
+      <x:c r="P23" s="10"/>
+      <x:c r="Q23" s="10"/>
+      <x:c r="R23" s="10"/>
+      <x:c r="S23" s="10"/>
+      <x:c r="T23" s="10"/>
+      <x:c r="U23" s="10"/>
+    </x:row>
+    <x:row r="24" ht="60" customHeight="1">
+      <x:c r="A24" s="165" t="str">
+        <x:v>Stage 7: Deep-site operations</x:v>
+      </x:c>
+      <x:c r="B24" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C24" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D24" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E24" s="169" t="n">
+        <x:f>MAX(0,D24)*(30*'Campaign Scenarios'!$B$18+'Campaign Scenarios'!$B$21)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F24" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G24" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H24" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I24" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J24" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K24" s="169" t="n">
+        <x:f>SUM(B24:C24)+E24+F24+G24*H24+I24+J24</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L24" s="170" t="str">
+        <x:v>VGE is optional; delivered vehicles stay physical. Base site fee is included.</x:v>
+      </x:c>
+      <x:c r="M24" s="10"/>
+      <x:c r="N24" s="10"/>
+      <x:c r="O24" s="10"/>
+      <x:c r="P24" s="10"/>
+      <x:c r="Q24" s="10"/>
+      <x:c r="R24" s="10"/>
+      <x:c r="S24" s="10"/>
+      <x:c r="T24" s="10"/>
+      <x:c r="U24" s="10"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="10"/>
+      <x:c r="B25" s="10"/>
+      <x:c r="C25" s="10"/>
+      <x:c r="D25" s="10"/>
+      <x:c r="E25" s="10"/>
+      <x:c r="F25" s="10"/>
+      <x:c r="G25" s="10"/>
+      <x:c r="H25" s="10"/>
+      <x:c r="I25" s="10"/>
+      <x:c r="J25" s="10"/>
+      <x:c r="K25" s="10"/>
+      <x:c r="L25" s="10"/>
+      <x:c r="M25" s="10"/>
+      <x:c r="N25" s="10"/>
+      <x:c r="O25" s="10"/>
+      <x:c r="P25" s="10"/>
+      <x:c r="Q25" s="10"/>
+      <x:c r="R25" s="10"/>
+      <x:c r="S25" s="10"/>
+      <x:c r="T25" s="10"/>
+      <x:c r="U25" s="10"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="10"/>
+      <x:c r="B26" s="10"/>
+      <x:c r="C26" s="10"/>
+      <x:c r="D26" s="10"/>
+      <x:c r="E26" s="10"/>
+      <x:c r="F26" s="10"/>
+      <x:c r="G26" s="10"/>
+      <x:c r="H26" s="10"/>
+      <x:c r="I26" s="10"/>
+      <x:c r="J26" s="10"/>
+      <x:c r="K26" s="10"/>
+      <x:c r="L26" s="10"/>
+      <x:c r="M26" s="10"/>
+      <x:c r="N26" s="10"/>
+      <x:c r="O26" s="10"/>
+      <x:c r="P26" s="10"/>
+      <x:c r="Q26" s="10"/>
+      <x:c r="R26" s="10"/>
+      <x:c r="S26" s="10"/>
+      <x:c r="T26" s="10"/>
+      <x:c r="U26" s="10"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="351" t="str">
+        <x:v>Long expedition extension beyond the 30-day base case</x:v>
+      </x:c>
+      <x:c r="B27" s="351"/>
+      <x:c r="C27" s="351"/>
+      <x:c r="D27" s="351"/>
+      <x:c r="E27" s="351"/>
+      <x:c r="F27" s="351"/>
+      <x:c r="G27" s="351"/>
+      <x:c r="H27" s="351"/>
+      <x:c r="I27" s="351"/>
+      <x:c r="J27" s="351"/>
+      <x:c r="K27" s="351"/>
+      <x:c r="L27" s="351"/>
+      <x:c r="M27" s="351"/>
+      <x:c r="N27" s="10"/>
+      <x:c r="O27" s="10"/>
+      <x:c r="P27" s="10"/>
+      <x:c r="Q27" s="10"/>
+      <x:c r="R27" s="10"/>
+      <x:c r="S27" s="10"/>
+      <x:c r="T27" s="10"/>
+      <x:c r="U27" s="10"/>
+    </x:row>
+    <x:row r="28" ht="66" customHeight="1">
+      <x:c r="A28" s="353" t="str">
+        <x:v>Campaign stage</x:v>
+      </x:c>
+      <x:c r="B28" s="353" t="str">
+        <x:v>Additional expedition days</x:v>
+      </x:c>
+      <x:c r="C28" s="353" t="str">
+        <x:v>Field crew count</x:v>
+      </x:c>
+      <x:c r="D28" s="353" t="str">
+        <x:v>Extra specialist premium / crew / day (USD)</x:v>
+      </x:c>
+      <x:c r="E28" s="353" t="str">
+        <x:v>Provision/support invoice / person-day (USD)</x:v>
+      </x:c>
+      <x:c r="F28" s="353" t="str">
+        <x:v>Extended base payroll (USD)</x:v>
+      </x:c>
+      <x:c r="G28" s="353" t="str">
+        <x:v>Extended specialist premium (USD)</x:v>
+      </x:c>
+      <x:c r="H28" s="353" t="str">
+        <x:v>Physical provisions/support quote (USD)</x:v>
+      </x:c>
+      <x:c r="I28" s="353" t="str">
+        <x:v>Transport/fuel/return quote (USD)</x:v>
+      </x:c>
+      <x:c r="J28" s="353" t="str">
+        <x:v>Equipment/consumable replacement (USD)</x:v>
+      </x:c>
+      <x:c r="K28" s="353" t="str">
+        <x:v>Rescue/evacuation reserve (USD)</x:v>
+      </x:c>
+      <x:c r="L28" s="353" t="str">
+        <x:v>Total extension cost (USD)</x:v>
+      </x:c>
+      <x:c r="M28" s="353" t="str">
+        <x:v>Basis / status</x:v>
+      </x:c>
+      <x:c r="N28" s="10"/>
+      <x:c r="O28" s="10"/>
+      <x:c r="P28" s="10"/>
+      <x:c r="Q28" s="10"/>
+      <x:c r="R28" s="10"/>
+      <x:c r="S28" s="10"/>
+      <x:c r="T28" s="10"/>
+      <x:c r="U28" s="10"/>
+    </x:row>
+    <x:row r="29" ht="60" customHeight="1">
+      <x:c r="A29" s="313" t="str">
+        <x:v>Stage 1: First safe survey</x:v>
+      </x:c>
+      <x:c r="B29" s="365" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C29" s="365" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D29" s="366" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E29" s="366" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F29" s="310" t="n">
+        <x:f>MAX(0,B29)*MAX(0,C29)*'Economy'!$C$34</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G29" s="310" t="n">
+        <x:f>MAX(0,B29)*MAX(0,C29)*MAX(0,D29)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H29" s="310" t="n">
+        <x:f>MAX(0,B29)*MAX(0,C29)*MAX(0,E29)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I29" s="366" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J29" s="366" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K29" s="366" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L29" s="310" t="n">
+        <x:f>SUM(F29:K29)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M29" s="301" t="str">
+        <x:v>Beyond day 30 only; supplies stay physical. Avoid duplicate quotes.</x:v>
+      </x:c>
+      <x:c r="N29" s="10"/>
+      <x:c r="O29" s="10"/>
+      <x:c r="P29" s="10"/>
+      <x:c r="Q29" s="10"/>
+      <x:c r="R29" s="10"/>
+      <x:c r="S29" s="10"/>
+      <x:c r="T29" s="10"/>
+      <x:c r="U29" s="10"/>
+    </x:row>
+    <x:row r="30" ht="60" customHeight="1">
+      <x:c r="A30" s="165" t="str">
+        <x:v>Stage 2: Repeat access</x:v>
+      </x:c>
+      <x:c r="B30" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C30" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D30" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E30" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F30" s="169" t="n">
+        <x:f>MAX(0,B30)*MAX(0,C30)*'Campaign Scenarios'!$B$18</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G30" s="169" t="n">
+        <x:f>MAX(0,B30)*MAX(0,C30)*MAX(0,D30)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H30" s="169" t="n">
+        <x:f>MAX(0,B30)*MAX(0,C30)*MAX(0,E30)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I30" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J30" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K30" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L30" s="169" t="n">
+        <x:f>SUM(F30:K30)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M30" s="170" t="str">
+        <x:v>Beyond day 30 only; supplies stay physical. Avoid duplicate quotes.</x:v>
+      </x:c>
+      <x:c r="N30" s="10"/>
+      <x:c r="O30" s="10"/>
+      <x:c r="P30" s="10"/>
+      <x:c r="Q30" s="10"/>
+      <x:c r="R30" s="10"/>
+      <x:c r="S30" s="10"/>
+      <x:c r="T30" s="10"/>
+      <x:c r="U30" s="10"/>
+    </x:row>
+    <x:row r="31" ht="60" customHeight="1">
+      <x:c r="A31" s="165" t="str">
+        <x:v>Stage 3: Specialist services</x:v>
+      </x:c>
+      <x:c r="B31" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C31" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D31" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E31" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F31" s="169" t="n">
+        <x:f>MAX(0,B31)*MAX(0,C31)*'Campaign Scenarios'!$B$18</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G31" s="169" t="n">
+        <x:f>MAX(0,B31)*MAX(0,C31)*MAX(0,D31)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H31" s="169" t="n">
+        <x:f>MAX(0,B31)*MAX(0,C31)*MAX(0,E31)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I31" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J31" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K31" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L31" s="169" t="n">
+        <x:f>SUM(F31:K31)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M31" s="170" t="str">
+        <x:v>Beyond day 30 only; supplies stay physical. Avoid duplicate quotes.</x:v>
+      </x:c>
+      <x:c r="N31" s="10"/>
+      <x:c r="O31" s="10"/>
+      <x:c r="P31" s="10"/>
+      <x:c r="Q31" s="10"/>
+      <x:c r="R31" s="10"/>
+      <x:c r="S31" s="10"/>
+      <x:c r="T31" s="10"/>
+      <x:c r="U31" s="10"/>
+    </x:row>
+    <x:row r="32" ht="60" customHeight="1">
+      <x:c r="A32" s="165" t="str">
+        <x:v>Stage 4: Leases and remote sites</x:v>
+      </x:c>
+      <x:c r="B32" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C32" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D32" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E32" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F32" s="169" t="n">
+        <x:f>MAX(0,B32)*MAX(0,C32)*'Campaign Scenarios'!$B$18</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G32" s="169" t="n">
+        <x:f>MAX(0,B32)*MAX(0,C32)*MAX(0,D32)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H32" s="169" t="n">
+        <x:f>MAX(0,B32)*MAX(0,C32)*MAX(0,E32)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I32" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J32" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K32" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L32" s="169" t="n">
+        <x:f>SUM(F32:K32)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M32" s="170" t="str">
+        <x:v>Beyond day 30 only; supplies stay physical. Avoid duplicate quotes.</x:v>
+      </x:c>
+      <x:c r="N32" s="10"/>
+      <x:c r="O32" s="10"/>
+      <x:c r="P32" s="10"/>
+      <x:c r="Q32" s="10"/>
+      <x:c r="R32" s="10"/>
+      <x:c r="S32" s="10"/>
+      <x:c r="T32" s="10"/>
+      <x:c r="U32" s="10"/>
+    </x:row>
+    <x:row r="33" ht="60" customHeight="1">
+      <x:c r="A33" s="165" t="str">
+        <x:v>Stage 5: Large recovery and network work</x:v>
+      </x:c>
+      <x:c r="B33" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C33" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D33" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E33" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F33" s="169" t="n">
+        <x:f>MAX(0,B33)*MAX(0,C33)*'Campaign Scenarios'!$B$18</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G33" s="169" t="n">
+        <x:f>MAX(0,B33)*MAX(0,C33)*MAX(0,D33)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H33" s="169" t="n">
+        <x:f>MAX(0,B33)*MAX(0,C33)*MAX(0,E33)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I33" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J33" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K33" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L33" s="169" t="n">
+        <x:f>SUM(F33:K33)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M33" s="170" t="str">
+        <x:v>Beyond day 30 only; supplies stay physical. Avoid duplicate quotes.</x:v>
+      </x:c>
+      <x:c r="N33" s="10"/>
+      <x:c r="O33" s="10"/>
+      <x:c r="P33" s="10"/>
+      <x:c r="Q33" s="10"/>
+      <x:c r="R33" s="10"/>
+      <x:c r="S33" s="10"/>
+      <x:c r="T33" s="10"/>
+      <x:c r="U33" s="10"/>
+    </x:row>
+    <x:row r="34" ht="60" customHeight="1">
+      <x:c r="A34" s="165" t="str">
+        <x:v>Stage 6: Vehicle and optional orbital support</x:v>
+      </x:c>
+      <x:c r="B34" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C34" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D34" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E34" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F34" s="169" t="n">
+        <x:f>MAX(0,B34)*MAX(0,C34)*'Campaign Scenarios'!$B$18</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G34" s="169" t="n">
+        <x:f>MAX(0,B34)*MAX(0,C34)*MAX(0,D34)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H34" s="169" t="n">
+        <x:f>MAX(0,B34)*MAX(0,C34)*MAX(0,E34)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I34" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J34" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K34" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L34" s="169" t="n">
+        <x:f>SUM(F34:K34)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M34" s="170" t="str">
+        <x:v>Beyond day 30 only; supplies stay physical. Avoid duplicate quotes.</x:v>
+      </x:c>
+      <x:c r="N34" s="10"/>
+      <x:c r="O34" s="10"/>
+      <x:c r="P34" s="10"/>
+      <x:c r="Q34" s="10"/>
+      <x:c r="R34" s="10"/>
+      <x:c r="S34" s="10"/>
+      <x:c r="T34" s="10"/>
+      <x:c r="U34" s="10"/>
+    </x:row>
+    <x:row r="35" ht="60" customHeight="1">
+      <x:c r="A35" s="165" t="str">
+        <x:v>Stage 7: Deep-site operations</x:v>
+      </x:c>
+      <x:c r="B35" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C35" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D35" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E35" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F35" s="169" t="n">
+        <x:f>MAX(0,B35)*MAX(0,C35)*'Campaign Scenarios'!$B$18</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G35" s="169" t="n">
+        <x:f>MAX(0,B35)*MAX(0,C35)*MAX(0,D35)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H35" s="169" t="n">
+        <x:f>MAX(0,B35)*MAX(0,C35)*MAX(0,E35)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I35" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J35" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K35" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L35" s="169" t="n">
+        <x:f>SUM(F35:K35)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M35" s="170" t="str">
+        <x:v>Beyond day 30 only; supplies stay physical. Avoid duplicate quotes.</x:v>
+      </x:c>
+      <x:c r="N35" s="10"/>
+      <x:c r="O35" s="10"/>
+      <x:c r="P35" s="10"/>
+      <x:c r="Q35" s="10"/>
+      <x:c r="R35" s="10"/>
+      <x:c r="S35" s="10"/>
+      <x:c r="T35" s="10"/>
+      <x:c r="U35" s="10"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="10"/>
+      <x:c r="B36" s="10"/>
+      <x:c r="C36" s="10"/>
+      <x:c r="D36" s="10"/>
+      <x:c r="E36" s="10"/>
+      <x:c r="F36" s="10"/>
+      <x:c r="G36" s="10"/>
+      <x:c r="H36" s="10"/>
+      <x:c r="I36" s="10"/>
+      <x:c r="J36" s="10"/>
+      <x:c r="K36" s="10"/>
+      <x:c r="L36" s="10"/>
+      <x:c r="M36" s="10"/>
+      <x:c r="N36" s="10"/>
+      <x:c r="O36" s="10"/>
+      <x:c r="P36" s="10"/>
+      <x:c r="Q36" s="10"/>
+      <x:c r="R36" s="10"/>
+      <x:c r="S36" s="10"/>
+      <x:c r="T36" s="10"/>
+      <x:c r="U36" s="10"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="10"/>
+      <x:c r="B37" s="10"/>
+      <x:c r="C37" s="10"/>
+      <x:c r="D37" s="10"/>
+      <x:c r="E37" s="10"/>
+      <x:c r="F37" s="10"/>
+      <x:c r="G37" s="10"/>
+      <x:c r="H37" s="10"/>
+      <x:c r="I37" s="10"/>
+      <x:c r="J37" s="10"/>
+      <x:c r="K37" s="10"/>
+      <x:c r="L37" s="10"/>
+      <x:c r="M37" s="10"/>
+      <x:c r="N37" s="10"/>
+      <x:c r="O37" s="10"/>
+      <x:c r="P37" s="10"/>
+      <x:c r="Q37" s="10"/>
+      <x:c r="R37" s="10"/>
+      <x:c r="S37" s="10"/>
+      <x:c r="T37" s="10"/>
+      <x:c r="U37" s="10"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="351" t="str">
+        <x:v>No-contract recovery: costs still committed and receipts actually realized</x:v>
+      </x:c>
+      <x:c r="B38" s="351"/>
+      <x:c r="C38" s="351"/>
+      <x:c r="D38" s="351"/>
+      <x:c r="E38" s="351"/>
+      <x:c r="F38" s="351"/>
+      <x:c r="G38" s="351"/>
+      <x:c r="H38" s="351"/>
+      <x:c r="I38" s="351"/>
+      <x:c r="J38" s="351"/>
+      <x:c r="K38" s="351"/>
+      <x:c r="L38" s="351"/>
+      <x:c r="M38" s="351"/>
+      <x:c r="N38" s="351"/>
+      <x:c r="O38" s="351"/>
+      <x:c r="P38" s="351"/>
+      <x:c r="Q38" s="351"/>
+      <x:c r="R38" s="351"/>
+      <x:c r="S38" s="351"/>
+      <x:c r="T38" s="351"/>
+      <x:c r="U38" s="351"/>
+    </x:row>
+    <x:row r="39" ht="72" customHeight="1">
+      <x:c r="A39" s="353" t="str">
+        <x:v>Campaign stage</x:v>
+      </x:c>
+      <x:c r="B39" s="353" t="str">
+        <x:v>Penalty contracts still due (count)</x:v>
+      </x:c>
+      <x:c r="C39" s="353" t="str">
+        <x:v>Penalty claimed per contract (USD)</x:v>
+      </x:c>
+      <x:c r="D39" s="353" t="str">
+        <x:v>Average contract value cap basis (USD)</x:v>
+      </x:c>
+      <x:c r="E39" s="353" t="str">
+        <x:v>Capped penalty still due (USD)</x:v>
+      </x:c>
+      <x:c r="F39" s="353" t="str">
+        <x:v>Cargo/crew response and rescue still due (USD)</x:v>
+      </x:c>
+      <x:c r="G39" s="353" t="str">
+        <x:v>Replacement orders still committed (USD)</x:v>
+      </x:c>
+      <x:c r="H39" s="353" t="str">
+        <x:v>Vehicle/gravship commitment still due (USD)</x:v>
+      </x:c>
+      <x:c r="I39" s="353" t="str">
+        <x:v>Additional outpost hires outside retained payroll (FTE)</x:v>
+      </x:c>
+      <x:c r="J39" s="353" t="str">
+        <x:v>Outpost security/defense due (USD)</x:v>
+      </x:c>
+      <x:c r="K39" s="353" t="str">
+        <x:v>Outpost resupply shipments due (count)</x:v>
+      </x:c>
+      <x:c r="L39" s="353" t="str">
+        <x:v>Invoice per shipment (USD)</x:v>
+      </x:c>
+      <x:c r="M39" s="353" t="str">
+        <x:v>Additional communications due (USD)</x:v>
+      </x:c>
+      <x:c r="N39" s="353" t="str">
+        <x:v>Outpost evacuation/closure reserve due (USD)</x:v>
+      </x:c>
+      <x:c r="O39" s="353" t="str">
+        <x:v>Long expedition extension still committed (USD)</x:v>
+      </x:c>
+      <x:c r="P39" s="353" t="str">
+        <x:v>Service receipts actually collected in recovery (USD)</x:v>
+      </x:c>
+      <x:c r="Q39" s="353" t="str">
+        <x:v>Lease receipts actually earned in recovery (USD)</x:v>
+      </x:c>
+      <x:c r="R39" s="353" t="str">
+        <x:v>Accepted claim reimbursement collected (USD)</x:v>
+      </x:c>
+      <x:c r="S39" s="353" t="str">
+        <x:v>Total recovery additions cost (USD)</x:v>
+      </x:c>
+      <x:c r="T39" s="353" t="str">
+        <x:v>Total recovery receipts (USD)</x:v>
+      </x:c>
+      <x:c r="U39" s="353" t="str">
+        <x:v>Basis / status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="60" customHeight="1">
+      <x:c r="A40" s="313" t="str">
+        <x:v>Stage 1: First safe survey</x:v>
+      </x:c>
+      <x:c r="B40" s="369" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C40" s="366" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D40" s="310" t="n">
+        <x:f>J7</x:f>
+        <x:v>5000000</x:v>
+      </x:c>
+      <x:c r="E40" s="310" t="n">
+        <x:f>MAX(0,B40)*MIN(MAX(0,C40),MAX(0,D40)*25%)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F40" s="366" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G40" s="366" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H40" s="366" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I40" s="365" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J40" s="366" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K40" s="365" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L40" s="366" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M40" s="366" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N40" s="366" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O40" s="366" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P40" s="366" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q40" s="366" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R40" s="366" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S40" s="310" t="n">
+        <x:f>E40+F40+G40+H40+MAX(0,I40)*(30*'Economy'!$C$34+'Economy'!$C$45)+J40+K40*L40+M40+N40+O40</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T40" s="310" t="n">
+        <x:f>SUM(P40:R40)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U40" s="301" t="str">
+        <x:v>Enter binding commitments only. Payroll remains on Recovery &amp; Capital.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="60" customHeight="1">
+      <x:c r="A41" s="165" t="str">
+        <x:v>Stage 2: Repeat access</x:v>
+      </x:c>
+      <x:c r="B41" s="370" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C41" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D41" s="169" t="n">
+        <x:f>J8</x:f>
+        <x:v>2500000</x:v>
+      </x:c>
+      <x:c r="E41" s="169" t="n">
+        <x:f>MAX(0,B41)*MIN(MAX(0,C41),MAX(0,D41)*25%)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F41" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G41" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H41" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I41" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J41" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K41" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L41" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M41" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N41" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O41" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P41" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q41" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R41" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S41" s="169" t="n">
+        <x:f>E41+F41+G41+H41+MAX(0,I41)*(30*'Campaign Scenarios'!$B$18+'Campaign Scenarios'!$B$21)+J41+K41*L41+M41+N41+O41</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T41" s="169" t="n">
+        <x:f>SUM(P41:R41)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U41" s="170" t="str">
+        <x:v>Enter binding commitments only. Payroll remains on Recovery &amp; Capital.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="60" customHeight="1">
+      <x:c r="A42" s="165" t="str">
+        <x:v>Stage 3: Specialist services</x:v>
+      </x:c>
+      <x:c r="B42" s="370" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C42" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D42" s="169" t="n">
+        <x:f>J9</x:f>
+        <x:v>10000000</x:v>
+      </x:c>
+      <x:c r="E42" s="169" t="n">
+        <x:f>MAX(0,B42)*MIN(MAX(0,C42),MAX(0,D42)*25%)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F42" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G42" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H42" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I42" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J42" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K42" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L42" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M42" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N42" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O42" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P42" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q42" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R42" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S42" s="169" t="n">
+        <x:f>E42+F42+G42+H42+MAX(0,I42)*(30*'Campaign Scenarios'!$B$18+'Campaign Scenarios'!$B$21)+J42+K42*L42+M42+N42+O42</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T42" s="169" t="n">
+        <x:f>SUM(P42:R42)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U42" s="170" t="str">
+        <x:v>Enter binding commitments only. Payroll remains on Recovery &amp; Capital.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="60" customHeight="1">
+      <x:c r="A43" s="165" t="str">
+        <x:v>Stage 4: Leases and remote sites</x:v>
+      </x:c>
+      <x:c r="B43" s="370" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C43" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D43" s="169" t="n">
+        <x:f>J10</x:f>
+        <x:v>25000000</x:v>
+      </x:c>
+      <x:c r="E43" s="169" t="n">
+        <x:f>MAX(0,B43)*MIN(MAX(0,C43),MAX(0,D43)*25%)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F43" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G43" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H43" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I43" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J43" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K43" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L43" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M43" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N43" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O43" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P43" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q43" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R43" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S43" s="169" t="n">
+        <x:f>E43+F43+G43+H43+MAX(0,I43)*(30*'Campaign Scenarios'!$B$18+'Campaign Scenarios'!$B$21)+J43+K43*L43+M43+N43+O43</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T43" s="169" t="n">
+        <x:f>SUM(P43:R43)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U43" s="170" t="str">
+        <x:v>Enter binding commitments only. Payroll remains on Recovery &amp; Capital.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="60" customHeight="1">
+      <x:c r="A44" s="165" t="str">
+        <x:v>Stage 5: Large recovery and network work</x:v>
+      </x:c>
+      <x:c r="B44" s="370" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C44" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D44" s="169" t="n">
+        <x:f>J11</x:f>
+        <x:v>75000000</x:v>
+      </x:c>
+      <x:c r="E44" s="169" t="n">
+        <x:f>MAX(0,B44)*MIN(MAX(0,C44),MAX(0,D44)*25%)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F44" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G44" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H44" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I44" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J44" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K44" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L44" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M44" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N44" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O44" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P44" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q44" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R44" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S44" s="169" t="n">
+        <x:f>E44+F44+G44+H44+MAX(0,I44)*(30*'Campaign Scenarios'!$B$18+'Campaign Scenarios'!$B$21)+J44+K44*L44+M44+N44+O44</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T44" s="169" t="n">
+        <x:f>SUM(P44:R44)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U44" s="170" t="str">
+        <x:v>Enter binding commitments only. Payroll remains on Recovery &amp; Capital.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="60" customHeight="1">
+      <x:c r="A45" s="165" t="str">
+        <x:v>Stage 6: Vehicle and optional orbital support</x:v>
+      </x:c>
+      <x:c r="B45" s="370" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C45" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D45" s="169" t="n">
+        <x:f>J12</x:f>
+        <x:v>150000000</x:v>
+      </x:c>
+      <x:c r="E45" s="169" t="n">
+        <x:f>MAX(0,B45)*MIN(MAX(0,C45),MAX(0,D45)*25%)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F45" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G45" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H45" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I45" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J45" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K45" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L45" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M45" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N45" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O45" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P45" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q45" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R45" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S45" s="169" t="n">
+        <x:f>E45+F45+G45+H45+MAX(0,I45)*(30*'Campaign Scenarios'!$B$18+'Campaign Scenarios'!$B$21)+J45+K45*L45+M45+N45+O45</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T45" s="169" t="n">
+        <x:f>SUM(P45:R45)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U45" s="170" t="str">
+        <x:v>Enter binding commitments only. Payroll remains on Recovery &amp; Capital.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="60" customHeight="1">
+      <x:c r="A46" s="165" t="str">
+        <x:v>Stage 7: Deep-site operations</x:v>
+      </x:c>
+      <x:c r="B46" s="370" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C46" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D46" s="169" t="n">
+        <x:f>J13</x:f>
+        <x:v>300000000</x:v>
+      </x:c>
+      <x:c r="E46" s="169" t="n">
+        <x:f>MAX(0,B46)*MIN(MAX(0,C46),MAX(0,D46)*25%)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F46" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G46" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H46" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I46" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J46" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K46" s="362" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L46" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M46" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N46" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O46" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P46" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q46" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="R46" s="361" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S46" s="169" t="n">
+        <x:f>E46+F46+G46+H46+MAX(0,I46)*(30*'Campaign Scenarios'!$B$18+'Campaign Scenarios'!$B$21)+J46+K46*L46+M46+N46+O46</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T46" s="169" t="n">
+        <x:f>SUM(P46:R46)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U46" s="170" t="str">
+        <x:v>Enter binding commitments only. Payroll remains on Recovery &amp; Capital.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>